<commit_message>
Implement MKB1 IR2 Batch 2 provisional waste cluster
</commit_message>
<xml_diff>
--- a/audit/mkb1-ontology-reuse-alignment/MKB1_IR2_Implementation_Tracker_2026-08-31 (2)_working implementation.xlsx
+++ b/audit/mkb1-ontology-reuse-alignment/MKB1_IR2_Implementation_Tracker_2026-08-31 (2)_working implementation.xlsx
@@ -1174,43 +1174,43 @@
       </c>
       <c r="I2" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J2" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/CollectionSystem</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000014</t>
         </is>
       </c>
       <c r="K2" s="33" t="inlineStr">
         <is>
-          <t>CollectionSystem: ACCEPT PROVISIONALLY — appropriate if the intended system is a material aggregate; hierarchy should be revisited when member, agent, function or realized-process queries become central.</t>
+          <t>CollectionSystem: ACCEPT PROVISIONALLY — implemented as an object aggregate; revisit member, agent, function, and realized-process modelling when those queries become central.</t>
         </is>
       </c>
       <c r="L2" s="33" t="inlineStr">
         <is>
-          <t>For now: CollectionSystem SubClassOf BFO object aggregate.</t>
+          <t>MATSUS_0000014 SubClassOf BFO_0000027.</t>
         </is>
       </c>
       <c r="M2" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N2" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O2" s="33" t="n"/>
       <c r="P2" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q2" s="33" t="inlineStr">
         <is>
-          <t>Reminder: recheck the hierarchy and LOG alignment when component, agent, function or realized-process queries become important.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R2" s="33" t="inlineStr">
@@ -1442,43 +1442,43 @@
       </c>
       <c r="I5" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J5" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/SortingProcess | https://w3id.org/pmd/matsus/SortingMethodSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000016 | https://w3id.org/pmd/matsus/MATSUS_0000017</t>
         </is>
       </c>
       <c r="K5" s="33" t="inlineStr">
         <is>
-          <t>SortingProcess: ACCEPT — generic sorting is correctly represented as a process. | SortingMethodSpecification: ACCEPT — correctly modelled as an information artifact, explicitly not as a sorting-process subclass.</t>
+          <t>SortingProcess: ACCEPT — implemented as a planned process. | SortingMethodSpecification: ACCEPT — implemented as an IAO plan specification and explicitly not as a SortingProcess subclass.</t>
         </is>
       </c>
       <c r="L5" s="33" t="inlineStr">
         <is>
-          <t>SortingProcess SubClassOf COB planned process. | SortingMethodSpecification SubClassOf IAO plan specification. No subclass axiom to SortingProcess.</t>
+          <t>MATSUS_0000016 SubClassOf COB_0000082. | MATSUS_0000017 SubClassOf IAO_0000104. No subclass axiom from MATSUS_0000017 to MATSUS_0000016.</t>
         </is>
       </c>
       <c r="M5" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N5" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O5" s="33" t="n"/>
       <c r="P5" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q5" s="33" t="inlineStr">
         <is>
-          <t>Connect process to method/plan during axiomatization; keep waste separation as a sorting-process subtype.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R5" s="33" t="inlineStr">
@@ -2854,12 +2854,12 @@
       </c>
       <c r="I21" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J21" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ConstructionAndDemolitionWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000009</t>
         </is>
       </c>
       <c r="K21" s="33" t="inlineStr">
@@ -2874,12 +2874,12 @@
       </c>
       <c r="M21" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N21" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O21" s="33" t="inlineStr">
@@ -2889,12 +2889,12 @@
       </c>
       <c r="P21" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q21" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R21" s="33" t="inlineStr">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
-          <t>waste-or-pollution elimination objective specification</t>
+          <t>waste elimination objective specification</t>
         </is>
       </c>
       <c r="E22" s="33" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="G22" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteOrPollutionEliminationObjectiveSpecification</t>
+          <t>https://w3id.org/pmd/matsus/WasteEliminationObjectiveSpecification</t>
         </is>
       </c>
       <c r="H22" s="33" t="inlineStr">
@@ -2946,32 +2946,32 @@
       </c>
       <c r="I22" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J22" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteOrPollutionEliminationObjectiveSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000024</t>
         </is>
       </c>
       <c r="K22" s="33" t="inlineStr">
         <is>
-          <t>WasteOrPollutionEliminationObjectiveSpecification: ACCEPT PROVISIONALLY — objective-specification modelling is correct; pollution still needs an independently scoped target entity/pattern.</t>
+          <t>WasteEliminationObjectiveSpecification: ACCEPT PROVISIONALLY — implemented for intended absence of specified waste output within a stated scope; pollution-elimination modelling is deferred.</t>
         </is>
       </c>
       <c r="L22" s="33" t="inlineStr">
         <is>
-          <t>WasteOrPollutionEliminationObjectiveSpecification SubClassOf IAO objective specification.</t>
+          <t>MATSUS_0000024 SubClassOf IAO_0000005.</t>
         </is>
       </c>
       <c r="M22" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N22" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O22" s="33" t="inlineStr">
@@ -2981,12 +2981,12 @@
       </c>
       <c r="P22" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q22" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Implemented for waste elimination only. Retain MKB-000085 provenance; defer pollution-elimination modelling until a suitable pollution target pattern is established.</t>
         </is>
       </c>
       <c r="R22" s="33" t="inlineStr">
@@ -3038,12 +3038,12 @@
       </c>
       <c r="I23" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J23" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MineralWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000010</t>
         </is>
       </c>
       <c r="K23" s="33" t="inlineStr">
@@ -3058,12 +3058,12 @@
       </c>
       <c r="M23" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N23" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O23" s="33" t="inlineStr">
@@ -3073,12 +3073,12 @@
       </c>
       <c r="P23" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q23" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R23" s="33" t="inlineStr">
@@ -3130,12 +3130,12 @@
       </c>
       <c r="I24" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J24" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MunicipalWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000011</t>
         </is>
       </c>
       <c r="K24" s="33" t="inlineStr">
@@ -3150,12 +3150,12 @@
       </c>
       <c r="M24" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N24" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O24" s="33" t="inlineStr">
@@ -3165,12 +3165,12 @@
       </c>
       <c r="P24" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q24" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R24" s="33" t="inlineStr">
@@ -3222,17 +3222,17 @@
       </c>
       <c r="I25" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J25" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/PackagingWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000012</t>
         </is>
       </c>
       <c r="K25" s="33" t="inlineStr">
         <is>
-          <t>PackagingWaste: REVISE BEFORE MERGE — parent is correct; definition should be aligned explicitly with the selected packaging-waste source and its exclusions.</t>
+          <t>PackagingWaste: ACCEPT — implemented with the selected source-aligned definition; production-residue exclusion remains an editorial constraint pending a validated logical pattern.</t>
         </is>
       </c>
       <c r="L25" s="33" t="inlineStr">
@@ -3242,12 +3242,12 @@
       </c>
       <c r="M25" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N25" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O25" s="33" t="inlineStr">
@@ -3257,12 +3257,12 @@
       </c>
       <c r="P25" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q25" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R25" s="33" t="inlineStr">
@@ -3314,32 +3314,32 @@
       </c>
       <c r="I26" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J26" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteAnalysis | https://w3id.org/pmd/matsus/StructuralWasteAnalysis</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000025 | https://w3id.org/pmd/matsus/MATSUS_0000026</t>
         </is>
       </c>
       <c r="K26" s="33" t="inlineStr">
         <is>
-          <t>WasteAnalysis: ACCEPT — analysis as an assay producing information is the right pattern. | StructuralWasteAnalysis: REVISE BEFORE MERGE — parent is correct, but the draft definition mixes structural/compositional analysis with recurring-source analysis; narrow the definition or rename the class.</t>
+          <t>WasteAnalysis: ACCEPT — implemented as an OBI assay. | StructuralWasteAnalysis: ACCEPT — definition narrowed to composition, organization, or distribution of material constituents; recurring-source analysis is deferred as a sibling.</t>
         </is>
       </c>
       <c r="L26" s="33" t="inlineStr">
         <is>
-          <t>WasteAnalysis SubClassOf OBI assay. | StructuralWasteAnalysis SubClassOf WasteAnalysis.</t>
+          <t>MATSUS_0000025 SubClassOf OBI_0000070. | MATSUS_0000026 SubClassOf MATSUS_0000025.</t>
         </is>
       </c>
       <c r="M26" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N26" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O26" s="33" t="inlineStr">
@@ -3349,12 +3349,12 @@
       </c>
       <c r="P26" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q26" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R26" s="33" t="inlineStr">
@@ -3406,12 +3406,12 @@
       </c>
       <c r="I27" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J27" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/TextileWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000013</t>
         </is>
       </c>
       <c r="K27" s="33" t="inlineStr">
@@ -3426,12 +3426,12 @@
       </c>
       <c r="M27" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N27" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O27" s="33" t="inlineStr">
@@ -3441,12 +3441,12 @@
       </c>
       <c r="P27" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q27" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R27" s="33" t="inlineStr">
@@ -3498,12 +3498,12 @@
       </c>
       <c r="I28" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J28" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteGenerationProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000019</t>
         </is>
       </c>
       <c r="K28" s="33" t="inlineStr">
@@ -3513,17 +3513,17 @@
       </c>
       <c r="L28" s="33" t="inlineStr">
         <is>
-          <t>WasteGenerationProcess SubClassOf BFO process; has output some WasteMaterial (RO_0002234).</t>
+          <t>MATSUS_0000019 SubClassOf BFO_0000015; MATSUS_0000019 SubClassOf RO_0002234 some MATSUS_0000008.</t>
         </is>
       </c>
       <c r="M28" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N28" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O28" s="33" t="inlineStr">
@@ -3533,12 +3533,12 @@
       </c>
       <c r="P28" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q28" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R28" s="33" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="I29" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J29" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WastePreventionProcess | https://w3id.org/pmd/matsus/WastePreventionMeasureSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000020 | https://w3id.org/pmd/matsus/MATSUS_0000021</t>
         </is>
       </c>
       <c r="K29" s="33" t="inlineStr">
@@ -3610,12 +3610,12 @@
       </c>
       <c r="M29" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N29" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O29" s="33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="P29" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q29" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R29" s="33" t="inlineStr">
@@ -3682,12 +3682,12 @@
       </c>
       <c r="I30" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 2)</t>
         </is>
       </c>
       <c r="J30" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ZeroWasteObjectiveSpecification | https://w3id.org/pmd/matsus/ZeroWasteStrategySpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000022 | https://w3id.org/pmd/matsus/MATSUS_0000023</t>
         </is>
       </c>
       <c r="K30" s="33" t="inlineStr">
@@ -3702,12 +3702,12 @@
       </c>
       <c r="M30" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 2</t>
         </is>
       </c>
       <c r="N30" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
         </is>
       </c>
       <c r="O30" s="33" t="inlineStr">
@@ -3717,12 +3717,12 @@
       </c>
       <c r="P30" s="33" t="inlineStr">
         <is>
-          <t>PROVISIONAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q30" s="33" t="inlineStr">
         <is>
-          <t>Implement now in MatSus using provisional WasteRole/WasteMaterial anchors. If PMDco later accepts equivalent anchors, migrate/reconcile mappings, parents and restrictions; do not delete the MatSus specializations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R30" s="33" t="inlineStr">
@@ -4833,7 +4833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:Q46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4850,6 +4850,9 @@
     <col width="34" customWidth="1" min="12" max="12"/>
     <col width="48.4140625" customWidth="1" min="13" max="13"/>
     <col width="32.58203125" customWidth="1" min="14" max="14"/>
+    <col width="62" customWidth="1" min="15" max="15"/>
+    <col width="54" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4923,6 +4926,21 @@
           <t>Editorial note</t>
         </is>
       </c>
+      <c r="O1" s="41" t="inlineStr">
+        <is>
+          <t>Source / provenance</t>
+        </is>
+      </c>
+      <c r="P1" s="41" t="inlineStr">
+        <is>
+          <t>integrationMethod</t>
+        </is>
+      </c>
+      <c r="Q1" s="41" t="inlineStr">
+        <is>
+          <t>Validation status</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="33" t="inlineStr">
@@ -4942,7 +4960,7 @@
       </c>
       <c r="D2" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteRole</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000007</t>
         </is>
       </c>
       <c r="E2" s="33" t="inlineStr">
@@ -4952,7 +4970,7 @@
       </c>
       <c r="F2" s="33" t="inlineStr">
         <is>
-          <t>BFO role (BFO_0000023)</t>
+          <t>BFO role (http://purl.obolibrary.org/obo/BFO_0000023)</t>
         </is>
       </c>
       <c r="G2" s="33" t="inlineStr">
@@ -4967,12 +4985,12 @@
       </c>
       <c r="I2" s="33" t="inlineStr">
         <is>
-          <t>WasteRole SubClassOf BFO role.</t>
+          <t>MATSUS_0000007 SubClassOf BFO_0000023.</t>
         </is>
       </c>
       <c r="J2" s="33" t="inlineStr">
         <is>
-          <t>Later: decide realization/context relations and whether a PMDco class replaces this local anchor.</t>
+          <t>Later: decide realization/context relations and the future PMDco mapping.</t>
         </is>
       </c>
       <c r="K2" s="33" t="inlineStr">
@@ -4982,11 +5000,30 @@
       </c>
       <c r="L2" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M2" s="33" t="n"/>
-      <c r="N2" s="33" t="n"/>
+      <c r="N2" s="33" t="inlineStr">
+        <is>
+          <t>Waste status is contextual and role-based, not an intrinsic material kind. Later PMDco acceptance triggers migration or reconciliation, not deletion.</t>
+        </is>
+      </c>
+      <c r="O2" s="33" t="inlineStr">
+        <is>
+          <t>Class Review row 2; human-gate Closure; PMDco issue #485.</t>
+        </is>
+      </c>
+      <c r="P2" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of BFO role</t>
+        </is>
+      </c>
+      <c r="Q2" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="33" t="inlineStr">
@@ -5006,7 +5043,7 @@
       </c>
       <c r="D3" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteMaterial</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000008</t>
         </is>
       </c>
       <c r="E3" s="33" t="inlineStr">
@@ -5016,7 +5053,7 @@
       </c>
       <c r="F3" s="33" t="inlineStr">
         <is>
-          <t>PMDco material (PMD_0000000)</t>
+          <t>PMDco material (https://w3id.org/pmd/co/PMD_0000000)</t>
         </is>
       </c>
       <c r="G3" s="33" t="inlineStr">
@@ -5031,12 +5068,12 @@
       </c>
       <c r="I3" s="33" t="inlineStr">
         <is>
-          <t>WasteMaterial SubClassOf PMDco material; WasteMaterial bears role some WasteRole (RO_0000087).</t>
+          <t>MATSUS_0000008 SubClassOf PMD_0000000; MATSUS_0000008 SubClassOf RO_0000087 some MATSUS_0000007.</t>
         </is>
       </c>
       <c r="J3" s="33" t="inlineStr">
         <is>
-          <t>Later: decide whether the role restriction remains necessary-only or becomes part of an equivalence; reconcile with #485.</t>
+          <t>Later: decide necessary-only versus equivalence and select a temporal/context model.</t>
         </is>
       </c>
       <c r="K3" s="33" t="inlineStr">
@@ -5046,11 +5083,30 @@
       </c>
       <c r="L3" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M3" s="33" t="n"/>
-      <c r="N3" s="33" t="n"/>
+      <c r="N3" s="33" t="inlineStr">
+        <is>
+          <t>Use 'waste' as an alternative label. RO_0000087 has the standard label 'has role'. Do not make recovered material a subclass of waste material. No equivalence axiom.</t>
+        </is>
+      </c>
+      <c r="O3" s="33" t="inlineStr">
+        <is>
+          <t>Class Review row 3; human-gate Closure; PMDco issue #485.</t>
+        </is>
+      </c>
+      <c r="P3" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of PMDco material with a necessary waste-role restriction</t>
+        </is>
+      </c>
+      <c r="Q3" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="33" t="inlineStr">
@@ -5070,7 +5126,7 @@
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ConstructionAndDemolitionWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000009</t>
         </is>
       </c>
       <c r="E4" s="33" t="inlineStr">
@@ -5080,7 +5136,7 @@
       </c>
       <c r="F4" s="33" t="inlineStr">
         <is>
-          <t>MatSus waste material</t>
+          <t>MatSus waste material (https://w3id.org/pmd/matsus/MATSUS_0000008)</t>
         </is>
       </c>
       <c r="G4" s="33" t="inlineStr">
@@ -5095,12 +5151,12 @@
       </c>
       <c r="I4" s="33" t="inlineStr">
         <is>
-          <t>ConstructionAndDemolitionWaste SubClassOf WasteMaterial.</t>
+          <t>MATSUS_0000009 SubClassOf MATSUS_0000008.</t>
         </is>
       </c>
       <c r="J4" s="33" t="inlineStr">
         <is>
-          <t>Later: add provenance/source criteria only if data integration requires them.</t>
+          <t>Later: add source/provenance criteria only if data integration requires them.</t>
         </is>
       </c>
       <c r="K4" s="33" t="inlineStr">
@@ -5110,11 +5166,30 @@
       </c>
       <c r="L4" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M4" s="33" t="n"/>
-      <c r="N4" s="33" t="n"/>
+      <c r="N4" s="33" t="inlineStr">
+        <is>
+          <t>Retain this local subtype after any upstream anchor migration.</t>
+        </is>
+      </c>
+      <c r="O4" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000063; SRC-001 Circular Berlin; Master Analysis row 52.</t>
+        </is>
+      </c>
+      <c r="P4" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of waste material</t>
+        </is>
+      </c>
+      <c r="Q4" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="33" t="inlineStr">
@@ -5134,7 +5209,7 @@
       </c>
       <c r="D5" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MineralWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000010</t>
         </is>
       </c>
       <c r="E5" s="33" t="inlineStr">
@@ -5144,7 +5219,7 @@
       </c>
       <c r="F5" s="33" t="inlineStr">
         <is>
-          <t>MatSus waste material</t>
+          <t>MatSus waste material (https://w3id.org/pmd/matsus/MATSUS_0000008)</t>
         </is>
       </c>
       <c r="G5" s="33" t="inlineStr">
@@ -5159,12 +5234,12 @@
       </c>
       <c r="I5" s="33" t="inlineStr">
         <is>
-          <t>MineralWaste SubClassOf WasteMaterial.</t>
+          <t>MATSUS_0000010 SubClassOf MATSUS_0000008.</t>
         </is>
       </c>
       <c r="J5" s="33" t="inlineStr">
         <is>
-          <t>Later: model composition/threshold criteria as data or a classification specification, not an unsupported OWL cutoff.</t>
+          <t>Later: represent thresholds through data or a classification specification.</t>
         </is>
       </c>
       <c r="K5" s="33" t="inlineStr">
@@ -5174,11 +5249,30 @@
       </c>
       <c r="L5" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M5" s="33" t="n"/>
-      <c r="N5" s="33" t="n"/>
+      <c r="N5" s="33" t="inlineStr">
+        <is>
+          <t>Predominantly is intentionally not assigned an OWL cutoff.</t>
+        </is>
+      </c>
+      <c r="O5" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000144; SRC-003 European Environment Agency; Master Analysis row 69.</t>
+        </is>
+      </c>
+      <c r="P5" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of waste material</t>
+        </is>
+      </c>
+      <c r="Q5" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="33" t="inlineStr">
@@ -5198,7 +5292,7 @@
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MunicipalWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000011</t>
         </is>
       </c>
       <c r="E6" s="33" t="inlineStr">
@@ -5208,7 +5302,7 @@
       </c>
       <c r="F6" s="33" t="inlineStr">
         <is>
-          <t>MatSus waste material</t>
+          <t>MatSus waste material (https://w3id.org/pmd/matsus/MATSUS_0000008)</t>
         </is>
       </c>
       <c r="G6" s="33" t="inlineStr">
@@ -5223,12 +5317,12 @@
       </c>
       <c r="I6" s="33" t="inlineStr">
         <is>
-          <t>MunicipalWaste SubClassOf WasteMaterial.</t>
+          <t>MATSUS_0000011 SubClassOf MATSUS_0000008.</t>
         </is>
       </c>
       <c r="J6" s="33" t="inlineStr">
         <is>
-          <t>Later: do not make municipal solid waste equivalent unless scope equivalence is confirmed.</t>
+          <t>Later: assert equivalence only if municipal-waste and municipal-solid-waste scopes are confirmed identical.</t>
         </is>
       </c>
       <c r="K6" s="33" t="inlineStr">
@@ -5238,11 +5332,30 @@
       </c>
       <c r="L6" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M6" s="33" t="n"/>
-      <c r="N6" s="33" t="n"/>
+      <c r="N6" s="33" t="inlineStr">
+        <is>
+          <t>Municipal solid waste is an alternative label, not an equivalent class.</t>
+        </is>
+      </c>
+      <c r="O6" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000148; SRC-003 European Environment Agency; Master Analysis row 71.</t>
+        </is>
+      </c>
+      <c r="P6" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of waste material</t>
+        </is>
+      </c>
+      <c r="Q6" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="33" t="inlineStr">
@@ -5262,17 +5375,17 @@
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/PackagingWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000012</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>A waste material that was packaging or packaging material before it acquired a waste role. Additional comment: this excludes production residues.</t>
+          <t>A waste material that was packaging or packaging material before it acquired a waste role.</t>
         </is>
       </c>
       <c r="F7" s="33" t="inlineStr">
         <is>
-          <t>MatSus waste material</t>
+          <t>MatSus waste material (https://w3id.org/pmd/matsus/MATSUS_0000008)</t>
         </is>
       </c>
       <c r="G7" s="33" t="inlineStr">
@@ -5287,12 +5400,12 @@
       </c>
       <c r="I7" s="33" t="inlineStr">
         <is>
-          <t>PackagingWaste SubClassOf WasteMaterial.</t>
+          <t>MATSUS_0000012 SubClassOf MATSUS_0000008.</t>
         </is>
       </c>
       <c r="J7" s="33" t="inlineStr">
         <is>
-          <t>Later: record former packaging function/role and any production-residue exclusion if required by the source definition.</t>
+          <t>Later: represent former packaging status and the production-residue exclusion only with a validated pattern.</t>
         </is>
       </c>
       <c r="K7" s="33" t="inlineStr">
@@ -5302,11 +5415,30 @@
       </c>
       <c r="L7" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M7" s="33" t="n"/>
-      <c r="N7" s="33" t="n"/>
+      <c r="N7" s="33" t="inlineStr">
+        <is>
+          <t>The selected source scope excludes production residues.</t>
+        </is>
+      </c>
+      <c r="O7" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000155; SRC-003 European Environment Agency; Master Analysis row 74; TransformON exact-label evidence was insufficient for reuse.</t>
+        </is>
+      </c>
+      <c r="P7" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of waste material</t>
+        </is>
+      </c>
+      <c r="Q7" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="33" t="inlineStr">
@@ -5326,7 +5458,7 @@
       </c>
       <c r="D8" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/TextileWaste</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000013</t>
         </is>
       </c>
       <c r="E8" s="33" t="inlineStr">
@@ -5336,7 +5468,7 @@
       </c>
       <c r="F8" s="33" t="inlineStr">
         <is>
-          <t>MatSus waste material</t>
+          <t>MatSus waste material (https://w3id.org/pmd/matsus/MATSUS_0000008)</t>
         </is>
       </c>
       <c r="G8" s="33" t="inlineStr">
@@ -5351,12 +5483,12 @@
       </c>
       <c r="I8" s="33" t="inlineStr">
         <is>
-          <t>TextileWaste SubClassOf WasteMaterial.</t>
+          <t>MATSUS_0000013 SubClassOf MATSUS_0000008.</t>
         </is>
       </c>
       <c r="J8" s="33" t="inlineStr">
         <is>
-          <t>Later: add fibre/composition/product-type refinements only from concrete use cases.</t>
+          <t>Later: add fibre, composition, or product-type refinements only from concrete use cases.</t>
         </is>
       </c>
       <c r="K8" s="33" t="inlineStr">
@@ -5366,11 +5498,30 @@
       </c>
       <c r="L8" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M8" s="33" t="n"/>
-      <c r="N8" s="33" t="n"/>
+      <c r="N8" s="33" t="inlineStr">
+        <is>
+          <t>Intentionally broad provisional subtype.</t>
+        </is>
+      </c>
+      <c r="O8" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000249; SRC-001 Circular Berlin; Master Analysis row 111.</t>
+        </is>
+      </c>
+      <c r="P8" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of waste material</t>
+        </is>
+      </c>
+      <c r="Q8" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="33" t="inlineStr">
@@ -5390,7 +5541,7 @@
       </c>
       <c r="D9" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteCollectionProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000015</t>
         </is>
       </c>
       <c r="E9" s="33" t="inlineStr">
@@ -5400,7 +5551,7 @@
       </c>
       <c r="F9" s="33" t="inlineStr">
         <is>
-          <t>COB planned process (COB_0000082)</t>
+          <t>COB planned process (http://purl.obolibrary.org/obo/COB_0000082)</t>
         </is>
       </c>
       <c r="G9" s="33" t="inlineStr">
@@ -5415,12 +5566,12 @@
       </c>
       <c r="I9" s="33" t="inlineStr">
         <is>
-          <t>WasteCollectionProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000015 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="J9" s="33" t="inlineStr">
         <is>
-          <t>Later: add waste participant, source location, destination and responsible-agent relations.</t>
+          <t>Later: add waste participant, origin, destination, and responsible-agent relations.</t>
         </is>
       </c>
       <c r="K9" s="33" t="inlineStr">
@@ -5430,11 +5581,30 @@
       </c>
       <c r="L9" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M9" s="33" t="n"/>
-      <c r="N9" s="33" t="n"/>
+      <c r="N9" s="33" t="inlineStr">
+        <is>
+          <t>Supporting process with no standalone MKB ID.</t>
+        </is>
+      </c>
+      <c r="O9" s="33" t="inlineStr">
+        <is>
+          <t>Class Review row 9; human-gate Closure related-terms decision.</t>
+        </is>
+      </c>
+      <c r="P9" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of COB planned process</t>
+        </is>
+      </c>
+      <c r="Q9" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="33" t="inlineStr">
@@ -5454,7 +5624,7 @@
       </c>
       <c r="D10" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/SortingProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000016</t>
         </is>
       </c>
       <c r="E10" s="33" t="inlineStr">
@@ -5464,7 +5634,7 @@
       </c>
       <c r="F10" s="33" t="inlineStr">
         <is>
-          <t>COB planned process (COB_0000082)</t>
+          <t>COB planned process (http://purl.obolibrary.org/obo/COB_0000082)</t>
         </is>
       </c>
       <c r="G10" s="33" t="inlineStr">
@@ -5479,22 +5649,41 @@
       </c>
       <c r="I10" s="33" t="inlineStr">
         <is>
-          <t>SortingProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000016 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="J10" s="33" t="inlineStr">
         <is>
-          <t>Later: connect the process to its criteria/method specification and sorted inputs/outputs.</t>
+          <t>Later: connect criteria/method specifications and sorted inputs/outputs.</t>
         </is>
       </c>
       <c r="K10" s="33" t="n"/>
       <c r="L10" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M10" s="33" t="n"/>
-      <c r="N10" s="33" t="n"/>
+      <c r="N10" s="33" t="inlineStr">
+        <is>
+          <t>Generic sorting is represented as a process.</t>
+        </is>
+      </c>
+      <c r="O10" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000231; SRC-001 Circular Berlin; Master Analysis row 106; no acceptable maintained equivalent found.</t>
+        </is>
+      </c>
+      <c r="P10" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of COB planned process</t>
+        </is>
+      </c>
+      <c r="Q10" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="33" t="inlineStr">
@@ -5514,7 +5703,7 @@
       </c>
       <c r="D11" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteSeparationProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000018</t>
         </is>
       </c>
       <c r="E11" s="33" t="inlineStr">
@@ -5524,7 +5713,7 @@
       </c>
       <c r="F11" s="33" t="inlineStr">
         <is>
-          <t>MatSus sorting process</t>
+          <t>MatSus sorting process (https://w3id.org/pmd/matsus/MATSUS_0000016)</t>
         </is>
       </c>
       <c r="G11" s="33" t="inlineStr">
@@ -5539,7 +5728,7 @@
       </c>
       <c r="I11" s="33" t="inlineStr">
         <is>
-          <t>WasteSeparationProcess SubClassOf SortingProcess.</t>
+          <t>MATSUS_0000018 SubClassOf MATSUS_0000016.</t>
         </is>
       </c>
       <c r="J11" s="33" t="inlineStr">
@@ -5554,11 +5743,30 @@
       </c>
       <c r="L11" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M11" s="33" t="n"/>
-      <c r="N11" s="33" t="n"/>
+      <c r="N11" s="33" t="inlineStr">
+        <is>
+          <t>Supporting process with no standalone MKB ID.</t>
+        </is>
+      </c>
+      <c r="O11" s="33" t="inlineStr">
+        <is>
+          <t>Class Review row 11; human-gate Closure related-terms decision.</t>
+        </is>
+      </c>
+      <c r="P11" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of sorting process</t>
+        </is>
+      </c>
+      <c r="Q11" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="33" t="inlineStr">
@@ -5578,7 +5786,7 @@
       </c>
       <c r="D12" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteGenerationProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000019</t>
         </is>
       </c>
       <c r="E12" s="33" t="inlineStr">
@@ -5588,7 +5796,7 @@
       </c>
       <c r="F12" s="33" t="inlineStr">
         <is>
-          <t>BFO process (BFO_0000015)</t>
+          <t>BFO process (http://purl.obolibrary.org/obo/BFO_0000015)</t>
         </is>
       </c>
       <c r="G12" s="33" t="inlineStr">
@@ -5603,12 +5811,12 @@
       </c>
       <c r="I12" s="33" t="inlineStr">
         <is>
-          <t>WasteGenerationProcess SubClassOf BFO process; has output some WasteMaterial (RO_0002234).</t>
+          <t>MATSUS_0000019 SubClassOf BFO_0000015; MATSUS_0000019 SubClassOf RO_0002234 some MATSUS_0000008.</t>
         </is>
       </c>
       <c r="J12" s="33" t="inlineStr">
         <is>
-          <t>Later: distinguish planned manufacturing waste from unplanned generation through context, not subclasses unless needed.</t>
+          <t>Later: distinguish planned and unplanned generation through context unless required otherwise.</t>
         </is>
       </c>
       <c r="K12" s="33" t="inlineStr">
@@ -5618,11 +5826,30 @@
       </c>
       <c r="L12" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M12" s="33" t="n"/>
-      <c r="N12" s="33" t="n"/>
+      <c r="N12" s="33" t="inlineStr">
+        <is>
+          <t>Generation is not assumed to be planned production or synthesis.</t>
+        </is>
+      </c>
+      <c r="O12" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000263; SRC-003 European Environment Agency; Master Analysis row 115.</t>
+        </is>
+      </c>
+      <c r="P12" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of BFO process with a necessary waste-material output restriction</t>
+        </is>
+      </c>
+      <c r="Q12" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="33" t="inlineStr">
@@ -5642,7 +5869,7 @@
       </c>
       <c r="D13" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WastePreventionProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000020</t>
         </is>
       </c>
       <c r="E13" s="33" t="inlineStr">
@@ -5652,7 +5879,7 @@
       </c>
       <c r="F13" s="33" t="inlineStr">
         <is>
-          <t>COB planned process (COB_0000082)</t>
+          <t>COB planned process (http://purl.obolibrary.org/obo/COB_0000082)</t>
         </is>
       </c>
       <c r="G13" s="33" t="inlineStr">
@@ -5667,12 +5894,12 @@
       </c>
       <c r="I13" s="33" t="inlineStr">
         <is>
-          <t>WastePreventionProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000020 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="J13" s="33" t="inlineStr">
         <is>
-          <t>Later: relate prevention processes to targeted material/product streams and prevention outcomes.</t>
+          <t>Later: relate the process to targeted streams and prevention outcomes.</t>
         </is>
       </c>
       <c r="K13" s="33" t="inlineStr">
@@ -5682,11 +5909,30 @@
       </c>
       <c r="L13" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M13" s="33" t="n"/>
-      <c r="N13" s="33" t="n"/>
+      <c r="N13" s="33" t="inlineStr">
+        <is>
+          <t>Keep the performed process distinct from its measure specification.</t>
+        </is>
+      </c>
+      <c r="O13" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000264; SRC-001 Circular Berlin; SRC-003 European Environment Agency; Master Analysis row 116.</t>
+        </is>
+      </c>
+      <c r="P13" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of COB planned process</t>
+        </is>
+      </c>
+      <c r="Q13" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="33" t="inlineStr">
@@ -5706,7 +5952,7 @@
       </c>
       <c r="D14" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WastePreventionMeasureSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000021</t>
         </is>
       </c>
       <c r="E14" s="33" t="inlineStr">
@@ -5716,7 +5962,7 @@
       </c>
       <c r="F14" s="33" t="inlineStr">
         <is>
-          <t>IAO plan specification (IAO_0000104)</t>
+          <t>IAO plan specification (http://purl.obolibrary.org/obo/IAO_0000104)</t>
         </is>
       </c>
       <c r="G14" s="33" t="inlineStr">
@@ -5731,12 +5977,12 @@
       </c>
       <c r="I14" s="33" t="inlineStr">
         <is>
-          <t>WastePreventionMeasureSpecification SubClassOf IAO plan specification.</t>
+          <t>MATSUS_0000021 SubClassOf IAO_0000104.</t>
         </is>
       </c>
       <c r="J14" s="33" t="inlineStr">
         <is>
-          <t>Later: connect the specification to the planned process it prescribes.</t>
+          <t>Later: connect it to the prescribed process.</t>
         </is>
       </c>
       <c r="K14" s="33" t="inlineStr">
@@ -5746,11 +5992,30 @@
       </c>
       <c r="L14" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M14" s="33" t="n"/>
-      <c r="N14" s="33" t="n"/>
+      <c r="N14" s="33" t="inlineStr">
+        <is>
+          <t>This is an information artifact, not a process.</t>
+        </is>
+      </c>
+      <c r="O14" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000264; SRC-001 Circular Berlin; SRC-003 European Environment Agency; Master Analysis row 116.</t>
+        </is>
+      </c>
+      <c r="P14" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO plan specification</t>
+        </is>
+      </c>
+      <c r="Q14" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="33" t="inlineStr">
@@ -5770,7 +6035,7 @@
       </c>
       <c r="D15" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ZeroWasteObjectiveSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000022</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr">
@@ -5780,7 +6045,7 @@
       </c>
       <c r="F15" s="33" t="inlineStr">
         <is>
-          <t>IAO objective specification (IAO_0000005)</t>
+          <t>IAO objective specification (http://purl.obolibrary.org/obo/IAO_0000005)</t>
         </is>
       </c>
       <c r="G15" s="33" t="inlineStr">
@@ -5795,12 +6060,12 @@
       </c>
       <c r="I15" s="33" t="inlineStr">
         <is>
-          <t>ZeroWasteObjectiveSpecification SubClassOf IAO objective specification.</t>
+          <t>MATSUS_0000022 SubClassOf IAO_0000005.</t>
         </is>
       </c>
       <c r="J15" s="33" t="inlineStr">
         <is>
-          <t>Later: represent scope, baseline and tolerated residual waste as information content if required.</t>
+          <t>Later: represent scope, baseline, and tolerated residual waste if needed.</t>
         </is>
       </c>
       <c r="K15" s="33" t="inlineStr">
@@ -5810,11 +6075,30 @@
       </c>
       <c r="L15" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M15" s="33" t="n"/>
-      <c r="N15" s="33" t="n"/>
+      <c r="N15" s="33" t="inlineStr">
+        <is>
+          <t>Zero waste is normative information content, not a material or process.</t>
+        </is>
+      </c>
+      <c r="O15" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000266; SRC-001 Circular Berlin; Master Analysis row 117.</t>
+        </is>
+      </c>
+      <c r="P15" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO objective specification</t>
+        </is>
+      </c>
+      <c r="Q15" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
@@ -5834,7 +6118,7 @@
       </c>
       <c r="D16" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ZeroWasteStrategySpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000023</t>
         </is>
       </c>
       <c r="E16" s="33" t="inlineStr">
@@ -5844,7 +6128,7 @@
       </c>
       <c r="F16" s="33" t="inlineStr">
         <is>
-          <t>IAO plan specification (IAO_0000104)</t>
+          <t>IAO plan specification (http://purl.obolibrary.org/obo/IAO_0000104)</t>
         </is>
       </c>
       <c r="G16" s="33" t="inlineStr">
@@ -5859,12 +6143,12 @@
       </c>
       <c r="I16" s="33" t="inlineStr">
         <is>
-          <t>ZeroWasteStrategySpecification SubClassOf IAO plan specification.</t>
+          <t>MATSUS_0000023 SubClassOf IAO_0000104.</t>
         </is>
       </c>
       <c r="J16" s="33" t="inlineStr">
         <is>
-          <t>Later: relate the strategy to its objective and prescribed prevention/reuse/recovery processes.</t>
+          <t>Later: relate it to the objective and prescribed prevention, reuse, and recovery processes.</t>
         </is>
       </c>
       <c r="K16" s="33" t="inlineStr">
@@ -5874,11 +6158,30 @@
       </c>
       <c r="L16" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M16" s="33" t="n"/>
-      <c r="N16" s="33" t="n"/>
+      <c r="N16" s="33" t="inlineStr">
+        <is>
+          <t>Keep the strategy distinct from its objective.</t>
+        </is>
+      </c>
+      <c r="O16" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000266; SRC-001 Circular Berlin; Master Analysis row 117.</t>
+        </is>
+      </c>
+      <c r="P16" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO plan specification</t>
+        </is>
+      </c>
+      <c r="Q16" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="33" t="inlineStr">
@@ -5898,7 +6201,7 @@
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteAnalysis</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000025</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
@@ -5908,7 +6211,7 @@
       </c>
       <c r="F17" s="33" t="inlineStr">
         <is>
-          <t>OBI assay (OBI_0000070)</t>
+          <t>OBI assay (http://purl.obolibrary.org/obo/OBI_0000070)</t>
         </is>
       </c>
       <c r="G17" s="33" t="inlineStr">
@@ -5923,12 +6226,12 @@
       </c>
       <c r="I17" s="33" t="inlineStr">
         <is>
-          <t>WasteAnalysis SubClassOf OBI assay.</t>
+          <t>MATSUS_0000025 SubClassOf OBI_0000070.</t>
         </is>
       </c>
       <c r="J17" s="33" t="inlineStr">
         <is>
-          <t>Later: add evaluant, method and output-datum relations using a concrete waste-stream example.</t>
+          <t>Later: add evaluant, method, and output-datum relations using a concrete example.</t>
         </is>
       </c>
       <c r="K17" s="33" t="inlineStr">
@@ -5938,11 +6241,30 @@
       </c>
       <c r="L17" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M17" s="33" t="n"/>
-      <c r="N17" s="33" t="n"/>
+      <c r="N17" s="33" t="inlineStr">
+        <is>
+          <t>Analysis is an assay, not the information output itself.</t>
+        </is>
+      </c>
+      <c r="O17" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000236; SRC-001 Circular Berlin; Master Analysis row 107.</t>
+        </is>
+      </c>
+      <c r="P17" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of OBI assay</t>
+        </is>
+      </c>
+      <c r="Q17" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="33" t="inlineStr">
@@ -5962,22 +6284,22 @@
       </c>
       <c r="D18" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/StructuralWasteAnalysis</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000026</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
         <is>
-          <t>A waste analysis intended to produce information about the composition, organization, distribution, or recurring generation patterns of a waste stream or waste-generating system.</t>
+          <t>A waste analysis intended to produce information about the composition, organization, or distribution of material constituents within a waste material or waste stream.</t>
         </is>
       </c>
       <c r="F18" s="33" t="inlineStr">
         <is>
-          <t>MatSus waste analysis</t>
+          <t>MatSus waste analysis (https://w3id.org/pmd/matsus/MATSUS_0000025)</t>
         </is>
       </c>
       <c r="G18" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACCEPT </t>
+          <t>ACCEPT — narrowed to composition, organization, or distribution of material constituents; recurring-source analysis is deferred as a sibling.</t>
         </is>
       </c>
       <c r="H18" s="33" t="inlineStr">
@@ -5987,12 +6309,12 @@
       </c>
       <c r="I18" s="33" t="inlineStr">
         <is>
-          <t>StructuralWasteAnalysis SubClassOf WasteAnalysis.</t>
+          <t>MATSUS_0000026 SubClassOf MATSUS_0000025.</t>
         </is>
       </c>
       <c r="J18" s="33" t="inlineStr">
         <is>
-          <t>Later: decide whether source analysis is a sibling of structural/composition analysis.</t>
+          <t>Later: consider recurring-source analysis as a deferred sibling class.</t>
         </is>
       </c>
       <c r="K18" s="33" t="inlineStr">
@@ -6002,15 +6324,34 @@
       </c>
       <c r="L18" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M18" s="33" t="inlineStr">
         <is>
-          <t>thoughts before resovling: dont get whats the problem with the draft definition mixes structural/compositional analysis with recurring-source analysis; narrow the definition or rename the class. cant it be generic? whats isdiffernet between structral waste analysis and waste anaylsis in matsus</t>
-        </is>
-      </c>
-      <c r="N18" s="33" t="n"/>
+          <t>thoughts before resovling: dont get whats the problem with the draft definition mixes structural/compositional analysis with recurring-source analysis; narrow the definition or rename the class. cant it be generic? whats isdiffernet between structral waste analysis and waste anaylsis in matsus Resolution: narrow StructuralWasteAnalysis and defer recurring-source analysis as a sibling.</t>
+        </is>
+      </c>
+      <c r="N18" s="33" t="inlineStr">
+        <is>
+          <t>Recurring-generation-pattern analysis is intentionally excluded from this definition.</t>
+        </is>
+      </c>
+      <c r="O18" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000236; SRC-001 Circular Berlin; Master Analysis row 107.</t>
+        </is>
+      </c>
+      <c r="P18" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of waste analysis</t>
+        </is>
+      </c>
+      <c r="Q18" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="33" t="inlineStr">
@@ -6090,7 +6431,7 @@
       </c>
       <c r="D20" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/SortingMethodSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000017</t>
         </is>
       </c>
       <c r="E20" s="33" t="inlineStr">
@@ -6100,7 +6441,7 @@
       </c>
       <c r="F20" s="33" t="inlineStr">
         <is>
-          <t>IAO plan specification (IAO_0000104)</t>
+          <t>IAO plan specification (http://purl.obolibrary.org/obo/IAO_0000104)</t>
         </is>
       </c>
       <c r="G20" s="33" t="inlineStr">
@@ -6115,7 +6456,7 @@
       </c>
       <c r="I20" s="33" t="inlineStr">
         <is>
-          <t>SortingMethodSpecification SubClassOf IAO plan specification. No subclass axiom to SortingProcess.</t>
+          <t>MATSUS_0000017 SubClassOf IAO_0000104. No subclass axiom to MATSUS_0000016.</t>
         </is>
       </c>
       <c r="J20" s="33" t="inlineStr">
@@ -6126,11 +6467,30 @@
       <c r="K20" s="33" t="n"/>
       <c r="L20" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M20" s="33" t="n"/>
-      <c r="N20" s="33" t="n"/>
+      <c r="N20" s="33" t="inlineStr">
+        <is>
+          <t>This is an information content entity and is not a subclass of SortingProcess.</t>
+        </is>
+      </c>
+      <c r="O20" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000231; SRC-001 Circular Berlin; Master Analysis row 106.</t>
+        </is>
+      </c>
+      <c r="P20" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO plan specification</t>
+        </is>
+      </c>
+      <c r="Q20" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="33" t="inlineStr">
@@ -6385,27 +6745,27 @@
       </c>
       <c r="C25" s="33" t="inlineStr">
         <is>
-          <t>waste or pollution elimination objective specification</t>
+          <t>waste elimination objective specification</t>
         </is>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/WasteOrPollutionEliminationObjectiveSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000024</t>
         </is>
       </c>
       <c r="E25" s="33" t="inlineStr">
         <is>
-          <t>An objective specification that describes an intended endpoint in which a specified waste or pollution output is absent.</t>
+          <t>An objective specification that specifies the intended absence of a specified waste output within a stated scope.</t>
         </is>
       </c>
       <c r="F25" s="33" t="inlineStr">
         <is>
-          <t>IAO objective specification (IAO_0000005)</t>
+          <t>IAO objective specification (http://purl.obolibrary.org/obo/IAO_0000005)</t>
         </is>
       </c>
       <c r="G25" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT PROVISIONALLY — objective-specification modelling is correct; pollution still needs an independently scoped target entity/pattern.</t>
+          <t>ACCEPT PROVISIONALLY — objective-specification modelling is correct; pollution-elimination modelling remains deferred pending a suitable target pattern.</t>
         </is>
       </c>
       <c r="H25" s="33" t="inlineStr">
@@ -6415,12 +6775,12 @@
       </c>
       <c r="I25" s="33" t="inlineStr">
         <is>
-          <t>WasteOrPollutionEliminationObjectiveSpecification SubClassOf IAO objective specification.</t>
+          <t>MATSUS_0000024 SubClassOf IAO_0000005.</t>
         </is>
       </c>
       <c r="J25" s="33" t="inlineStr">
         <is>
-          <t>Later: link to the specified waste/pollution target and boundary; do not mint an undefined generic elimination process.</t>
+          <t>Later: link to a scoped waste target and boundary. Pollution-elimination modelling is deferred until a suitable pollution target pattern is established.</t>
         </is>
       </c>
       <c r="K25" s="33" t="inlineStr">
@@ -6430,11 +6790,30 @@
       </c>
       <c r="L25" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M25" s="33" t="n"/>
-      <c r="N25" s="33" t="n"/>
+      <c r="N25" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000085 is retained as provenance. Do not create a generic elimination process or pollution class.</t>
+        </is>
+      </c>
+      <c r="O25" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000085; SRC-002 Ellen MacArthur Foundation; Master Analysis row 56.</t>
+        </is>
+      </c>
+      <c r="P25" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO objective specification</t>
+        </is>
+      </c>
+      <c r="Q25" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="33" t="inlineStr">
@@ -7134,7 +7513,7 @@
       </c>
       <c r="D37" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/CollectionSystem</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000014</t>
         </is>
       </c>
       <c r="E37" s="33" t="inlineStr">
@@ -7144,7 +7523,7 @@
       </c>
       <c r="F37" s="33" t="inlineStr">
         <is>
-          <t>BFO object aggregate (BFO_0000027)</t>
+          <t>BFO object aggregate (http://purl.obolibrary.org/obo/BFO_0000027)</t>
         </is>
       </c>
       <c r="G37" s="33" t="inlineStr">
@@ -7159,22 +7538,41 @@
       </c>
       <c r="I37" s="33" t="inlineStr">
         <is>
-          <t>For now: CollectionSystem SubClassOf BFO object aggregate.</t>
+          <t>MATSUS_0000014 SubClassOf BFO_0000027.</t>
         </is>
       </c>
       <c r="J37" s="33" t="inlineStr">
         <is>
-          <t>Later: model members/components, enabling function, responsible agent and collection processes; do not introduce a universal System class.</t>
+          <t>Later: model members/components, enabling function, responsible agent, and collection processes when those queries become central.</t>
         </is>
       </c>
       <c r="K37" s="33" t="n"/>
       <c r="L37" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 2)</t>
         </is>
       </c>
       <c r="M37" s="33" t="n"/>
-      <c r="N37" s="33" t="n"/>
+      <c r="N37" s="33" t="inlineStr">
+        <is>
+          <t>The object-aggregate parent is provisional. Do not introduce a universal generic System class.</t>
+        </is>
+      </c>
+      <c r="O37" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000059; IR2 Tracker row 2; Class Review row 37.</t>
+        </is>
+      </c>
+      <c r="P37" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of BFO object aggregate</t>
+        </is>
+      </c>
+      <c r="Q37" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-04 — syntax, import closure, ODK full build, ELK, local OWL 2 DL, IDs, declarations, parents, restrictions, imports, and four repository SPARQL rules pass; full-closure profile is identical to main baseline; DC rule and ROBOT warnings are baseline-explained.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="42" customHeight="1">
       <c r="A38" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Implement MKB1 IR2 Batch 3 non-waste classes
</commit_message>
<xml_diff>
--- a/audit/mkb1-ontology-reuse-alignment/MKB1_IR2_Implementation_Tracker_2026-08-31 (2)_working implementation.xlsx
+++ b/audit/mkb1-ontology-reuse-alignment/MKB1_IR2_Implementation_Tracker_2026-08-31 (2)_working implementation.xlsx
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>COUNTIF('IR2 Tracker'!A2:A42,"1 - LOCAL IMPLEMENTATION")</f>
+        <f>COUNTIF('IR2 Tracker'!A2:A43,"1 - LOCAL IMPLEMENTATION")</f>
         <v/>
       </c>
       <c r="C6" s="3" t="n"/>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF('IR2 Tracker'!M2:M42,"YES")</f>
+        <f>COUNTIF('IR2 Tracker'!M2:M43,"YES")</f>
         <v/>
       </c>
       <c r="C7" s="3" t="n"/>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>COUNTIF('IR2 Tracker'!A2:A42,"3 - DEFERRED")</f>
+        <f>COUNTIF('IR2 Tracker'!A2:A43,"3 - DEFERRED")</f>
         <v/>
       </c>
       <c r="C10" s="3" t="n"/>
@@ -1017,7 +1017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1262,55 +1262,55 @@
       </c>
       <c r="I3" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J3" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MetricSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000027</t>
         </is>
       </c>
       <c r="K3" s="33" t="inlineStr">
         <is>
-          <t>MetricSpecification: ACCEPT — a metric specification prescribes calculation inputs/methods; the resulting metric value remains a data item.</t>
+          <t>MetricSpecification: ACCEPT ? implemented as an IAO directive information entity; resulting metric values remain data items.</t>
         </is>
       </c>
       <c r="L3" s="33" t="inlineStr">
         <is>
-          <t>MetricSpecification SubClassOf IAO directive information entity.</t>
+          <t>MATSUS_0000027 SubClassOf IAO_0000033.</t>
         </is>
       </c>
       <c r="M3" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N3" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O3" s="33" t="n"/>
       <c r="P3" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q3" s="33" t="inlineStr">
         <is>
-          <t>Use MetricSpecification for indicator methods; keep values/results under IAO data item.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R3" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="33" t="inlineStr">
         <is>
-          <t>1 - LOCAL IMPLEMENTATION</t>
+          <t>2 - EXTERNAL HANDOFF</t>
         </is>
       </c>
       <c r="B4" s="33" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="E4" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENT_LOCAL_MATSUS_TERM</t>
+          <t>EXTERNAL_ISSUE_DEPENDENT</t>
         </is>
       </c>
       <c r="F4" s="33" t="inlineStr">
@@ -1350,32 +1350,32 @@
       </c>
       <c r="I4" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>NOT_IMPLEMENTED_BATCH_3</t>
         </is>
       </c>
       <c r="J4" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/CircularDesignSpecification</t>
+          <t>N/A ? no Batch 3 IRI allocated</t>
         </is>
       </c>
       <c r="K4" s="33" t="inlineStr">
         <is>
-          <t>CircularDesignSpecification: ACCEPT PROVISIONALLY — usable local specialization, but the current directive-only parent/definition may be too narrow if PMDco issue #488 adopts a descriptive-or-directive specification-document pattern.</t>
+          <t>CircularDesignSpecification: EXTERNAL_ISSUE_DEPENDENT ? await PMDco #488; reconsider locally only if the generic PMDco DesignSpecification proposal is rejected.</t>
         </is>
       </c>
       <c r="L4" s="33" t="inlineStr">
         <is>
-          <t>For now: CircularDesignSpecification SubClassOf IAO directive information entity.</t>
+          <t>No MatSus axiom in Batch 3.</t>
         </is>
       </c>
       <c r="M4" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N4" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O4" s="33" t="inlineStr">
@@ -1385,17 +1385,17 @@
       </c>
       <c r="P4" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_ISSUE_SUBMITTED</t>
+          <t>ISSUE_SUBMITTED</t>
         </is>
       </c>
       <c r="Q4" s="33" t="inlineStr">
         <is>
-          <t>PMDco issue #488 submitted for generic design specification. Keep the MatSus circular design specialization; reconcile its parent after the PMDco decision.</t>
+          <t>Await PMDco #488; do not mint a MatSus duplicate now.</t>
         </is>
       </c>
       <c r="R4" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Batch 3 exclusion confirmed; planning history retained.</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="33" t="inlineStr">
         <is>
-          <t>1 - LOCAL IMPLEMENTATION</t>
+          <t>2 - EXTERNAL HANDOFF</t>
         </is>
       </c>
       <c r="B6" s="33" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENT_LOCAL_MATSUS_PATTERN</t>
+          <t>EXTERNAL_ISSUE_DEPENDENT</t>
         </is>
       </c>
       <c r="F6" s="33" t="inlineStr">
@@ -1530,32 +1530,32 @@
       </c>
       <c r="I6" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>NOT_IMPLEMENTED_BATCH_3</t>
         </is>
       </c>
       <c r="J6" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/FeedstockRole</t>
+          <t>N/A ? no Batch 3 IRI allocated</t>
         </is>
       </c>
       <c r="K6" s="33" t="inlineStr">
         <is>
-          <t>FeedstockRole: ACCEPT PROVISIONALLY — role modelling is correct and the LOG parent is reasonable; PMDco issue #486 may provide the upstream class and require reconciliation.</t>
+          <t>FeedstockRole: EXTERNAL_ISSUE_DEPENDENT ? await PMDco #486; reuse upstream if accepted, otherwise reconsider a local MatSus class.</t>
         </is>
       </c>
       <c r="L6" s="33" t="inlineStr">
         <is>
-          <t>For now: FeedstockRole SubClassOf LOG material resource role.</t>
+          <t>No MatSus axiom in Batch 3.</t>
         </is>
       </c>
       <c r="M6" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N6" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O6" s="33" t="inlineStr">
@@ -1565,17 +1565,17 @@
       </c>
       <c r="P6" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_ISSUE_SUBMITTED</t>
+          <t>ISSUE_SUBMITTED</t>
         </is>
       </c>
       <c r="Q6" s="33" t="inlineStr">
         <is>
-          <t>PMDco issue #486 submitted for feedstock role. Keep the MatSus FeedstockRole draft for current use; reconcile its parent/mapping if PMDco adopts the role.</t>
+          <t>Await PMDco #486; do not mint a MatSus duplicate now.</t>
         </is>
       </c>
       <c r="R6" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Batch 3 exclusion confirmed; PMDco/LOG placement remains external.</t>
         </is>
       </c>
     </row>
@@ -1617,53 +1617,53 @@
       </c>
       <c r="H7" s="33" t="inlineStr">
         <is>
-          <t>MatSus resource efficiency datum</t>
+          <t>MatSus resource efficiency datum (MATSUS_0000028)</t>
         </is>
       </c>
       <c r="I7" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J7" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MaterialResourceEfficiencyDatum</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000029</t>
         </is>
       </c>
       <c r="K7" s="33" t="inlineStr">
         <is>
-          <t>MaterialResourceEfficiencyDatum: ACCEPT — clear material-input specialization.</t>
+          <t>MaterialResourceEfficiencyDatum: ACCEPT ? implemented as the material-input specialization of MATSUS_0000028.</t>
         </is>
       </c>
       <c r="L7" s="33" t="inlineStr">
         <is>
-          <t>MaterialResourceEfficiencyDatum SubClassOf ResourceEfficiencyDatum.</t>
+          <t>MATSUS_0000029 SubClassOf MATSUS_0000028.</t>
         </is>
       </c>
       <c r="M7" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N7" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O7" s="33" t="n"/>
       <c r="P7" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q7" s="33" t="inlineStr">
         <is>
-          <t>Record output/value, material input, method, boundary and time interval in the instance pattern.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R7" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="D8" s="33" t="inlineStr">
         <is>
-          <t>virgin material (implemented); non-virgin material deferred</t>
+          <t>virgin material</t>
         </is>
       </c>
       <c r="E8" s="33" t="inlineStr">
         <is>
-          <t>DEFER_MODELLING_USE_CASE</t>
+          <t>IMPLEMENT_LOCAL_MATSUS_TERM</t>
         </is>
       </c>
       <c r="F8" s="33" t="inlineStr">
@@ -1710,48 +1710,48 @@
       </c>
       <c r="I8" s="33" t="inlineStr">
         <is>
-          <t>PARTIALLY_IMPLEMENTED</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J8" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/VirginMaterial</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000030</t>
         </is>
       </c>
       <c r="K8" s="33" t="inlineStr">
         <is>
-          <t>VirginMaterial: REVISE BEFORE MERGE — parent is correct; definition needs an explicit authoritative source and clearer treatment of mixed virgin/recovered constituents. Do not define non-virgin material as its OWL complement.</t>
+          <t>VirginMaterial: ACCEPT ? implemented with the approved ISO-grounded positive definition; use existing MATSUS_0000003 SecondaryMaterial and no complement class.</t>
         </is>
       </c>
       <c r="L8" s="33" t="inlineStr">
         <is>
-          <t>VirginMaterial SubClassOf PMDco material.</t>
+          <t>MATSUS_0000030 SubClassOf PMD_0000000.</t>
         </is>
       </c>
       <c r="M8" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N8" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O8" s="33" t="n"/>
       <c r="P8" s="33" t="inlineStr">
         <is>
-          <t>PARTIAL_DRAFT_READY</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q8" s="33" t="inlineStr">
         <is>
-          <t>Use recycled/recovered-content assertions; revisit a positive SecondaryMaterial class with a composition competency query.</t>
+          <t>Use existing positive MATSUS_0000003 SecondaryMaterial; recovered-content, composition, and proportion axioms remain deferred.</t>
         </is>
       </c>
       <c r="R8" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -1793,53 +1793,53 @@
       </c>
       <c r="H9" s="33" t="inlineStr">
         <is>
-          <t>repurposing process</t>
+          <t>MatSus repurposing process (MATSUS_0000031)</t>
         </is>
       </c>
       <c r="I9" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J9" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/BatteryRepurposingProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000032</t>
         </is>
       </c>
       <c r="K9" s="33" t="inlineStr">
         <is>
-          <t>BatteryRepurposingProcess: ACCEPT — appropriate battery-specific specialization.</t>
+          <t>BatteryRepurposingProcess: ACCEPT ? implemented as the battery-specific specialization of MATSUS_0000031.</t>
         </is>
       </c>
       <c r="L9" s="33" t="inlineStr">
         <is>
-          <t>BatteryRepurposingProcess SubClassOf RepurposingProcess.</t>
+          <t>MATSUS_0000032 SubClassOf MATSUS_0000031.</t>
         </is>
       </c>
       <c r="M9" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N9" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O9" s="33" t="n"/>
       <c r="P9" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q9" s="33" t="inlineStr">
         <is>
-          <t>Use a battery second-life example to test participant and new-purpose relations.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R9" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -1886,48 +1886,48 @@
       </c>
       <c r="I10" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J10" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ResourceInputReductionProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000033</t>
         </is>
       </c>
       <c r="K10" s="33" t="inlineStr">
         <is>
-          <t>ResourceInputReductionProcess: REVISE BEFORE MERGE — parent is correct, but the draft phrase ‘used by another process’ is ambiguous. Define it directly through lower resource input relative to a stated baseline and comparable output.</t>
+          <t>ResourceInputReductionProcess: ACCEPT ? implemented as a planned process distinct from its assessment and objective specification.</t>
         </is>
       </c>
       <c r="L10" s="33" t="inlineStr">
         <is>
-          <t>ResourceInputReductionProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000033 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="M10" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N10" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O10" s="33" t="n"/>
       <c r="P10" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q10" s="33" t="inlineStr">
         <is>
-          <t>Test with a manufacturing example: process P2 uses less material/energy than baseline P1 under the same output specification.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R10" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -1974,48 +1974,48 @@
       </c>
       <c r="I11" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J11" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RefillProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000034</t>
         </is>
       </c>
       <c r="K11" s="33" t="inlineStr">
         <is>
-          <t>RefillProcess: ACCEPT — one generic process correctly consolidates at-home and on-the-go contexts.</t>
+          <t>RefillProcess: ACCEPT ? one generic class consolidates MKB-000181 and MKB-000182.</t>
         </is>
       </c>
       <c r="L11" s="33" t="inlineStr">
         <is>
-          <t>RefillProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000034 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="M11" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N11" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O11" s="33" t="n"/>
       <c r="P11" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q11" s="33" t="inlineStr">
         <is>
-          <t>Keep at-home as source context; add a context relation only when queries require it.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R11" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -2062,48 +2062,48 @@
       </c>
       <c r="I12" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J12" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RefillProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000034</t>
         </is>
       </c>
       <c r="K12" s="33" t="inlineStr">
         <is>
-          <t>RefillProcess: ACCEPT — one generic process correctly consolidates at-home and on-the-go contexts.</t>
+          <t>RefillProcess: ACCEPT ? one generic class consolidates MKB-000181 and MKB-000182.</t>
         </is>
       </c>
       <c r="L12" s="33" t="inlineStr">
         <is>
-          <t>RefillProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000034 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="M12" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N12" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O12" s="33" t="n"/>
       <c r="P12" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q12" s="33" t="inlineStr">
         <is>
-          <t>Keep away-from-home as source context; add a context relation only when queries require it.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R12" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -2150,48 +2150,48 @@
       </c>
       <c r="I13" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J13" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RefusalProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000035</t>
         </is>
       </c>
       <c r="K13" s="33" t="inlineStr">
         <is>
-          <t>RefusalProcess: ACCEPT — intentional refusal is appropriately a planned process rather than a bare verb class.</t>
+          <t>RefusalProcess: ACCEPT ? implemented as the actual intentional refusal occurrence, distinct from strategy and objective specifications.</t>
         </is>
       </c>
       <c r="L13" s="33" t="inlineStr">
         <is>
-          <t>RefusalProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000035 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="M13" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N13" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O13" s="33" t="n"/>
       <c r="P13" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q13" s="33" t="inlineStr">
         <is>
-          <t>Test with a user declining single-use packaging; add agent/object relations during axiomatization.</t>
+          <t>Keep RefusalProcess distinct from RefusalStrategySpecification; add no logical relation between them in Batch 3.</t>
         </is>
       </c>
       <c r="R13" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -2238,48 +2238,48 @@
       </c>
       <c r="I14" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J14" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RemanufacturingProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000036</t>
         </is>
       </c>
       <c r="K14" s="33" t="inlineStr">
         <is>
-          <t>RemanufacturingProcess: ACCEPT — process parent and restorative-performance definition are defensible.</t>
+          <t>RemanufacturingProcess: ACCEPT ? implemented as a planned restorative process.</t>
         </is>
       </c>
       <c r="L14" s="33" t="inlineStr">
         <is>
-          <t>RemanufacturingProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000036 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="M14" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N14" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O14" s="33" t="n"/>
       <c r="P14" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q14" s="33" t="inlineStr">
         <is>
-          <t>If a capability query later needs remanufacturability, evaluate direct reuse of AutomatCE AUTOMATCE_0010231; do not duplicate it now.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R14" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -2326,55 +2326,55 @@
       </c>
       <c r="I15" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J15" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RepurposingProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000031</t>
         </is>
       </c>
       <c r="K15" s="33" t="inlineStr">
         <is>
-          <t>RepurposingProcess: ACCEPT — the new-purpose distinction is captured clearly.</t>
+          <t>RepurposingProcess: ACCEPT ? implemented as a planned process with purpose relations deferred.</t>
         </is>
       </c>
       <c r="L15" s="33" t="inlineStr">
         <is>
-          <t>RepurposingProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000031 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="M15" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N15" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O15" s="33" t="n"/>
       <c r="P15" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q15" s="33" t="inlineStr">
         <is>
-          <t>Represent new intended purpose and prior intended purpose in a later relation/SHACL pattern.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R15" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="56" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
         <is>
-          <t>1 - LOCAL IMPLEMENTATION</t>
+          <t>3 - DEFERRED</t>
         </is>
       </c>
       <c r="B16" s="33" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="E16" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENT_LOCAL_MATSUS_TERM</t>
+          <t>DEFER_MODELLING_USE_CASE</t>
         </is>
       </c>
       <c r="F16" s="33" t="inlineStr">
@@ -2414,48 +2414,48 @@
       </c>
       <c r="I16" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>NOT_IMPLEMENTED_BATCH_3</t>
         </is>
       </c>
       <c r="J16" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MaterialFlowProcess | https://w3id.org/pmd/matsus/TextileMaterialFlowProcess</t>
+          <t>N/A ? no Batch 3 IRI allocated</t>
         </is>
       </c>
       <c r="K16" s="33" t="inlineStr">
         <is>
-          <t>MaterialFlowProcess: ACCEPT PROVISIONALLY — generic process parent is safe, but LOG alignment should be revisited before strengthening the hierarchy. | TextileMaterialFlowProcess: ACCEPT PROVISIONALLY — correct material-specific specialization of the provisional flow process.</t>
+          <t>MaterialFlowProcess and TextileMaterialFlowProcess: DEFER ? require dedicated LOG transport, material-location-change, logistics, and material-flow-datum analysis.</t>
         </is>
       </c>
       <c r="L16" s="33" t="inlineStr">
         <is>
-          <t>MaterialFlowProcess SubClassOf BFO process. | TextileMaterialFlowProcess SubClassOf MaterialFlowProcess.</t>
+          <t>No MatSus axioms in Batch 3.</t>
         </is>
       </c>
       <c r="M16" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N16" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O16" s="33" t="n"/>
       <c r="P16" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="Q16" s="33" t="inlineStr">
         <is>
-          <t>Ask LOG colleagues whether MaterialFlowProcess should move upstream after a supply-chain competency example is available.</t>
+          <t>Complete the LOG-boundary and process-versus-datum analysis before implementation.</t>
         </is>
       </c>
       <c r="R16" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Both candidate classes remain absent; TextileMaterialFlowProcess retains its unsettled parent.</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>decoupling</t>
+          <t>decoupling datum</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="G17" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/Decoupling</t>
+          <t>https://w3id.org/pmd/matsus/DecouplingDatum</t>
         </is>
       </c>
       <c r="H17" s="33" t="inlineStr">
@@ -2502,48 +2502,48 @@
       </c>
       <c r="I17" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_CANONICAL_DEFERRED_NARROWER</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J17" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/Decoupling</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000037</t>
         </is>
       </c>
       <c r="K17" s="33" t="inlineStr">
         <is>
-          <t>Decoupling: ACCEPT — the definition makes clear that the class records a comparative relationship; absolute decoupling remains correctly deferred.</t>
+          <t>DecouplingDatum: ACCEPT ? implemented as the established sustainability/resource-efficiency comparative data item, not a separation process.</t>
         </is>
       </c>
       <c r="L17" s="33" t="inlineStr">
         <is>
-          <t>Decoupling SubClassOf IAO data item.</t>
+          <t>MATSUS_0000037 SubClassOf IAO_0000027.</t>
         </is>
       </c>
       <c r="M17" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N17" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O17" s="33" t="n"/>
       <c r="P17" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q17" s="33" t="inlineStr">
         <is>
-          <t>Defer AbsoluteDecoupling until the ratio/baseline pattern is tested.</t>
+          <t>Defer absolute/relative classifications, indicators, calculation method, ratio, baseline, and temporal relations.</t>
         </is>
       </c>
       <c r="R17" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
       </c>
       <c r="D18" s="33" t="inlineStr">
         <is>
-          <t>decoupling</t>
+          <t>decoupling datum</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
@@ -2580,7 +2580,7 @@
       </c>
       <c r="G18" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/Decoupling</t>
+          <t>https://w3id.org/pmd/matsus/DecouplingDatum</t>
         </is>
       </c>
       <c r="H18" s="33" t="inlineStr">
@@ -2590,48 +2590,48 @@
       </c>
       <c r="I18" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J18" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/Decoupling</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000037</t>
         </is>
       </c>
       <c r="K18" s="33" t="inlineStr">
         <is>
-          <t>Decoupling: ACCEPT — the definition makes clear that the class records a comparative relationship; absolute decoupling remains correctly deferred.</t>
+          <t>DecouplingDatum: ACCEPT ? one class consolidates MKB-000002 and MKB-000069.</t>
         </is>
       </c>
       <c r="L18" s="33" t="inlineStr">
         <is>
-          <t>Decoupling SubClassOf IAO data item.</t>
+          <t>MATSUS_0000037 SubClassOf IAO_0000027.</t>
         </is>
       </c>
       <c r="M18" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N18" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O18" s="33" t="n"/>
       <c r="P18" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q18" s="33" t="inlineStr">
         <is>
-          <t>Test with one economic-output/resource-input time-series example.</t>
+          <t>Defer absolute/relative classifications, indicators, calculation method, ratio, baseline, and temporal relations.</t>
         </is>
       </c>
       <c r="R18" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -2678,48 +2678,48 @@
       </c>
       <c r="I19" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J19" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/Modularity</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000038</t>
         </is>
       </c>
       <c r="K19" s="33" t="inlineStr">
         <is>
-          <t>Modularity: ACCEPT — degree of modular organization is appropriately represented as a quality.</t>
+          <t>Modularity: ACCEPT ? implemented as a BFO quality, not an object aggregate.</t>
         </is>
       </c>
       <c r="L19" s="33" t="inlineStr">
         <is>
-          <t>Modularity SubClassOf BFO quality.</t>
+          <t>MATSUS_0000038 SubClassOf BFO_0000019.</t>
         </is>
       </c>
       <c r="M19" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N19" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O19" s="33" t="n"/>
       <c r="P19" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q19" s="33" t="inlineStr">
         <is>
-          <t>Add a measurement datum/method only when a modularity metric is selected.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R19" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -2766,48 +2766,48 @@
       </c>
       <c r="I20" s="33" t="inlineStr">
         <is>
-          <t>IMPLEMENTED_IN_MATSUS_EDIT</t>
+          <t>IMPLEMENTED_IN_MATSUS_EDIT (BATCH 3)</t>
         </is>
       </c>
       <c r="J20" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ResourceEfficiencyDatum</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000028</t>
         </is>
       </c>
       <c r="K20" s="33" t="inlineStr">
         <is>
-          <t>ResourceEfficiencyDatum: ACCEPT — the class is a calculated/result datum, not an intrinsic universal ‘efficiency’.</t>
+          <t>ResourceEfficiencyDatum: ACCEPT ? implemented as a calculated/result datum, not an intrinsic quality.</t>
         </is>
       </c>
       <c r="L20" s="33" t="inlineStr">
         <is>
-          <t>ResourceEfficiencyDatum SubClassOf IAO data item.</t>
+          <t>MATSUS_0000028 SubClassOf IAO_0000027.</t>
         </is>
       </c>
       <c r="M20" s="33" t="inlineStr">
         <is>
-          <t>NO - DRAFT ONLY</t>
+          <t>YES - MKB1 IR2 BATCH 3</t>
         </is>
       </c>
       <c r="N20" s="33" t="inlineStr">
         <is>
-          <t>FULL BUILD TODO</t>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
       <c r="O20" s="33" t="n"/>
       <c r="P20" s="33" t="inlineStr">
         <is>
-          <t>DRAFT_READY_FOR_IR2</t>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
         </is>
       </c>
       <c r="Q20" s="33" t="inlineStr">
         <is>
-          <t>Use material resource efficiency as a subtype and add energy/resource subtypes only from competency queries.</t>
+          <t>Ready for human pre-commit review; retain deferred modelling notes.</t>
         </is>
       </c>
       <c r="R20" s="33" t="inlineStr">
         <is>
-          <t>Full class-level definition, parent, confidence and later-axiom notes are in Class Review.</t>
+          <t>Full class-level definition, exact parent, provenance, integration method, editorial decision, and later-axiom notes are in Class Review.</t>
         </is>
       </c>
     </row>
@@ -4800,6 +4800,94 @@
       <c r="R42" s="33" t="inlineStr">
         <is>
           <t>Final numeric IRI allocated under repository policy. IAO objective specification parent resolved in the current import closure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="58" customHeight="1">
+      <c r="A43" s="33" t="inlineStr">
+        <is>
+          <t>1 - LOCAL IMPLEMENTATION</t>
+        </is>
+      </c>
+      <c r="B43" s="33" t="inlineStr">
+        <is>
+          <t>Human-gate refinement from MKB-000184 review</t>
+        </is>
+      </c>
+      <c r="C43" s="33" t="inlineStr">
+        <is>
+          <t>Information/specification</t>
+        </is>
+      </c>
+      <c r="D43" s="33" t="inlineStr">
+        <is>
+          <t>refusal strategy specification</t>
+        </is>
+      </c>
+      <c r="E43" s="33" t="inlineStr">
+        <is>
+          <t>HUMAN_GATE_MODELLING_REFINEMENT</t>
+        </is>
+      </c>
+      <c r="F43" s="33" t="inlineStr">
+        <is>
+          <t>MatSus</t>
+        </is>
+      </c>
+      <c r="G43" s="33" t="inlineStr">
+        <is>
+          <t>https://w3id.org/pmd/matsus/RefusalStrategySpecification</t>
+        </is>
+      </c>
+      <c r="H43" s="33" t="inlineStr">
+        <is>
+          <t>IAO plan specification (IAO_0000104)</t>
+        </is>
+      </c>
+      <c r="I43" s="33" t="inlineStr">
+        <is>
+          <t>HUMAN_GATE_ADDITION</t>
+        </is>
+      </c>
+      <c r="J43" s="33" t="inlineStr">
+        <is>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000039</t>
+        </is>
+      </c>
+      <c r="K43" s="33" t="inlineStr">
+        <is>
+          <t>RefusalStrategySpecification: ACCEPT ? implemented as a plan specification distinct from the actual refusal occurrence.</t>
+        </is>
+      </c>
+      <c r="L43" s="33" t="inlineStr">
+        <is>
+          <t>MATSUS_0000039 SubClassOf IAO_0000104. No logical relation to MATSUS_0000035 in Batch 3.</t>
+        </is>
+      </c>
+      <c r="M43" s="33" t="inlineStr">
+        <is>
+          <t>YES - MKB1 IR2 BATCH 3</t>
+        </is>
+      </c>
+      <c r="N43" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
+      <c r="O43" s="33" t="n"/>
+      <c r="P43" s="33" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED_VALIDATED_WITH_BASELINE_EXPLAINED_WARNINGS</t>
+        </is>
+      </c>
+      <c r="Q43" s="33" t="inlineStr">
+        <is>
+          <t>Ready for human pre-commit review; all process/specification and objective relations remain deferred.</t>
+        </is>
+      </c>
+      <c r="R43" s="33" t="inlineStr">
+        <is>
+          <t>Additional human-gate modelling refinement derived from the MKB-000184 review; not a seventeenth original source candidate. Full record is in Class Review row 47.</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -6371,7 +6459,7 @@
       </c>
       <c r="D19" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RefillProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000034</t>
         </is>
       </c>
       <c r="E19" s="33" t="inlineStr">
@@ -6381,12 +6469,12 @@
       </c>
       <c r="F19" s="33" t="inlineStr">
         <is>
-          <t>COB planned process (COB_0000082)</t>
+          <t>COB planned process (http://purl.obolibrary.org/obo/COB_0000082)</t>
         </is>
       </c>
       <c r="G19" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — one generic process correctly consolidates at-home and on-the-go contexts.</t>
+          <t>ACCEPT ? one generic process consolidates the two source rows.</t>
         </is>
       </c>
       <c r="H19" s="33" t="inlineStr">
@@ -6396,22 +6484,41 @@
       </c>
       <c r="I19" s="33" t="inlineStr">
         <is>
-          <t>RefillProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000034 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="J19" s="33" t="inlineStr">
         <is>
-          <t>Later: add container/device, refilled material and context relations only when queries require them.</t>
+          <t>Later: model container/device, refilled material, location, agent, and context relations.</t>
         </is>
       </c>
       <c r="K19" s="33" t="n"/>
       <c r="L19" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M19" s="33" t="n"/>
-      <c r="N19" s="33" t="n"/>
+      <c r="N19" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000181 and MKB-000182 are consolidated into this class; at-home and on-the-go are source contexts, not subclasses.</t>
+        </is>
+      </c>
+      <c r="O19" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000181 and MKB-000182; SRC-002 Ellen MacArthur Foundation; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P19" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of COB planned process</t>
+        </is>
+      </c>
+      <c r="Q19" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="33" t="inlineStr">
@@ -6510,7 +6617,7 @@
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RepurposingProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000031</t>
         </is>
       </c>
       <c r="E21" s="33" t="inlineStr">
@@ -6520,12 +6627,12 @@
       </c>
       <c r="F21" s="33" t="inlineStr">
         <is>
-          <t>COB planned process (COB_0000082)</t>
+          <t>COB planned process (http://purl.obolibrary.org/obo/COB_0000082)</t>
         </is>
       </c>
       <c r="G21" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — the new-purpose distinction is captured clearly.</t>
+          <t>ACCEPT ? the new-purpose distinction is captured clearly; no maintained compatible process class was verified.</t>
         </is>
       </c>
       <c r="H21" s="33" t="inlineStr">
@@ -6535,22 +6642,41 @@
       </c>
       <c r="I21" s="33" t="inlineStr">
         <is>
-          <t>RepurposingProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000031 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="J21" s="33" t="inlineStr">
         <is>
-          <t>Later: represent prior intended purpose, new intended purpose and affected product/component/material.</t>
+          <t>Later: represent prior purpose, new purpose, participants, inputs, and outputs.</t>
         </is>
       </c>
       <c r="K21" s="33" t="n"/>
       <c r="L21" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M21" s="33" t="n"/>
-      <c r="N21" s="33" t="n"/>
+      <c r="N21" s="33" t="inlineStr">
+        <is>
+          <t>No maintained compatible repurposing-process class was verified in the reviewed sources.</t>
+        </is>
+      </c>
+      <c r="O21" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000202; SRC-001 Circular Berlin; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P21" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of COB planned process</t>
+        </is>
+      </c>
+      <c r="Q21" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="33" t="inlineStr">
@@ -6570,7 +6696,7 @@
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/BatteryRepurposingProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000032</t>
         </is>
       </c>
       <c r="E22" s="33" t="inlineStr">
@@ -6580,12 +6706,12 @@
       </c>
       <c r="F22" s="33" t="inlineStr">
         <is>
-          <t>MatSus repurposing process</t>
+          <t>MatSus repurposing process (https://w3id.org/pmd/matsus/MATSUS_0000031)</t>
         </is>
       </c>
       <c r="G22" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — appropriate battery-specific specialization.</t>
+          <t>ACCEPT ? appropriate battery-specific specialization.</t>
         </is>
       </c>
       <c r="H22" s="33" t="inlineStr">
@@ -6595,22 +6721,41 @@
       </c>
       <c r="I22" s="33" t="inlineStr">
         <is>
-          <t>BatteryRepurposingProcess SubClassOf RepurposingProcess.</t>
+          <t>MATSUS_0000032 SubClassOf MATSUS_0000031.</t>
         </is>
       </c>
       <c r="J22" s="33" t="inlineStr">
         <is>
-          <t>Later: add battery participant and second-life/new-purpose relations from a use case.</t>
+          <t>Later: add battery-participant and second-life or new-purpose relations from an approved use case.</t>
         </is>
       </c>
       <c r="K22" s="33" t="n"/>
       <c r="L22" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M22" s="33" t="n"/>
-      <c r="N22" s="33" t="n"/>
+      <c r="N22" s="33" t="inlineStr">
+        <is>
+          <t>Battery participant and second-life/new-purpose relations remain deferred.</t>
+        </is>
+      </c>
+      <c r="O22" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000009; SRC-002 Ellen MacArthur Foundation; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P22" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of repurposing process</t>
+        </is>
+      </c>
+      <c r="Q22" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="33" t="inlineStr">
@@ -6630,7 +6775,7 @@
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RemanufacturingProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000036</t>
         </is>
       </c>
       <c r="E23" s="33" t="inlineStr">
@@ -6640,12 +6785,12 @@
       </c>
       <c r="F23" s="33" t="inlineStr">
         <is>
-          <t>COB planned process (COB_0000082)</t>
+          <t>COB planned process (http://purl.obolibrary.org/obo/COB_0000082)</t>
         </is>
       </c>
       <c r="G23" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — process parent and restorative-performance definition are defensible.</t>
+          <t>ACCEPT ? process parent and restorative-performance definition are defensible.</t>
         </is>
       </c>
       <c r="H23" s="33" t="inlineStr">
@@ -6655,22 +6800,41 @@
       </c>
       <c r="I23" s="33" t="inlineStr">
         <is>
-          <t>RemanufacturingProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000036 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="J23" s="33" t="inlineStr">
         <is>
-          <t>Later: model used input, retained identity/components, restorative operations and specified output state.</t>
+          <t>Later: model used input, retained identity or components, restorative operations, and specified output state.</t>
         </is>
       </c>
       <c r="K23" s="33" t="n"/>
       <c r="L23" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M23" s="33" t="n"/>
-      <c r="N23" s="33" t="n"/>
+      <c r="N23" s="33" t="inlineStr">
+        <is>
+          <t>The process remains distinct from the separate AutomatCE remanufacturability disposition candidate.</t>
+        </is>
+      </c>
+      <c r="O23" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000189; SRC-003 European Environment Agency; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P23" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of COB planned process</t>
+        </is>
+      </c>
+      <c r="Q23" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="76" customHeight="1">
       <c r="A24" s="33" t="inlineStr">
@@ -6685,27 +6849,27 @@
       </c>
       <c r="C24" s="33" t="inlineStr">
         <is>
-          <t>resource input reduction process</t>
+          <t>resource-input reduction process</t>
         </is>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ResourceInputReductionProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000033</t>
         </is>
       </c>
       <c r="E24" s="33" t="inlineStr">
         <is>
-          <t>A planned process intended to reduce the amount of material input used by a process or system.</t>
+          <t>A planned process intended to reduce the amount of material input used by a specified process or system.</t>
         </is>
       </c>
       <c r="F24" s="33" t="inlineStr">
         <is>
-          <t>COB planned process (COB_0000082)</t>
+          <t>COB planned process (http://purl.obolibrary.org/obo/COB_0000082)</t>
         </is>
       </c>
       <c r="G24" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — broad intentional intervention class; the process may reduce material input directly or by changing another process or system.</t>
+          <t>ACCEPT ? broad intentional intervention class, kept distinct from its assessment and objective specification.</t>
         </is>
       </c>
       <c r="H24" s="33" t="inlineStr">
@@ -6715,22 +6879,41 @@
       </c>
       <c r="I24" s="33" t="inlineStr">
         <is>
-          <t>ResourceInputReductionProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000033 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="J24" s="33" t="inlineStr">
         <is>
-          <t>Evaluate the reduction relative to a stated baseline under comparable conditions. Later: model affected process/system, material input, baseline and comparable output or function.</t>
+          <t>Later: model the affected process or system, material input, stated baseline, comparison conditions, and comparable output or function.</t>
         </is>
       </c>
       <c r="K24" s="33" t="n"/>
       <c r="L24" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M24" s="33" t="n"/>
-      <c r="N24" s="33" t="n"/>
+      <c r="N24" s="33" t="inlineStr">
+        <is>
+          <t>Keep this process distinct from MATSUS_0000005 resource-input reduction assessment and MATSUS_0000006 resource-input reduction objective specification.</t>
+        </is>
+      </c>
+      <c r="O24" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000180; SRC-001 Circular Berlin; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P24" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of COB planned process</t>
+        </is>
+      </c>
+      <c r="Q24" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="33" t="inlineStr">
@@ -6833,7 +7016,7 @@
       </c>
       <c r="D26" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/RefusalProcess</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000035</t>
         </is>
       </c>
       <c r="E26" s="33" t="inlineStr">
@@ -6843,12 +7026,12 @@
       </c>
       <c r="F26" s="33" t="inlineStr">
         <is>
-          <t>COB planned process (COB_0000082)</t>
+          <t>COB planned process (http://purl.obolibrary.org/obo/COB_0000082)</t>
         </is>
       </c>
       <c r="G26" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — intentional refusal is appropriately a planned process rather than a bare verb class.</t>
+          <t>ACCEPT ? actual intentional refusal occurrence, distinct from strategy and objective specifications.</t>
         </is>
       </c>
       <c r="H26" s="33" t="inlineStr">
@@ -6858,22 +7041,41 @@
       </c>
       <c r="I26" s="33" t="inlineStr">
         <is>
-          <t>RefusalProcess SubClassOf COB planned process.</t>
+          <t>MATSUS_0000035 SubClassOf COB_0000082.</t>
         </is>
       </c>
       <c r="J26" s="33" t="inlineStr">
         <is>
-          <t>Later: add agent, refused entity/service and avoidance objective relations.</t>
+          <t>Later: add agent, refused entity or service, and avoidance-objective relations. Do not add a logical relation to RefusalStrategySpecification in Batch 3.</t>
         </is>
       </c>
       <c r="K26" s="33" t="n"/>
       <c r="L26" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M26" s="33" t="n"/>
-      <c r="N26" s="33" t="n"/>
+      <c r="N26" s="33" t="inlineStr">
+        <is>
+          <t>RefusalProcess represents the actual intentional refusal occurrence. It does not represent the strategy specification or objective specification that motivates, enables, or encourages that occurrence.</t>
+        </is>
+      </c>
+      <c r="O26" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000184; SRC-001 Circular Berlin; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P26" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of COB planned process</t>
+        </is>
+      </c>
+      <c r="Q26" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="33" t="inlineStr">
@@ -6888,27 +7090,27 @@
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
-          <t>decoupling</t>
+          <t>decoupling datum</t>
         </is>
       </c>
       <c r="D27" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/Decoupling</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000037</t>
         </is>
       </c>
       <c r="E27" s="33" t="inlineStr">
         <is>
-          <t>A data item that records a comparative temporal relationship in which an economic or service output and an associated environmental pressure or resource input change at different rates.</t>
+          <t>A data item that records a comparison over a stated time interval in which the rate of change of a resource input or environmental pressure is lower than the rate of change of a specified economic or service output.</t>
         </is>
       </c>
       <c r="F27" s="33" t="inlineStr">
         <is>
-          <t>IAO data item (IAO_0000027)</t>
+          <t>IAO data item (http://purl.obolibrary.org/obo/IAO_0000027)</t>
         </is>
       </c>
       <c r="G27" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — the definition makes clear that the class records a comparative relationship; absolute decoupling remains correctly deferred.</t>
+          <t>ACCEPT ? established sustainability/resource-efficiency comparative datum, not a physical separation process.</t>
         </is>
       </c>
       <c r="H27" s="33" t="inlineStr">
@@ -6918,22 +7120,41 @@
       </c>
       <c r="I27" s="33" t="inlineStr">
         <is>
-          <t>Decoupling SubClassOf IAO data item.</t>
+          <t>MATSUS_0000037 SubClassOf IAO_0000027.</t>
         </is>
       </c>
       <c r="J27" s="33" t="inlineStr">
         <is>
-          <t>Later: represent economic/service output, pressure/resource input, baseline, time interval and comparison method.</t>
+          <t>Later: model absolute and relative classifications, baseline and comparison interval, resource-input or environmental-pressure indicator, economic or service-output indicator, calculation method, ratio, and temporal relations.</t>
         </is>
       </c>
       <c r="K27" s="33" t="n"/>
       <c r="L27" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M27" s="33" t="n"/>
-      <c r="N27" s="33" t="n"/>
+      <c r="N27" s="33" t="inlineStr">
+        <is>
+          <t>This records sustainability/resource-efficiency decoupling, not dismantling, disassembly, or another physical separation process.</t>
+        </is>
+      </c>
+      <c r="O27" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000002, SRC-003 European Environment Agency; MKB-000069, SRC-002 Ellen MacArthur Foundation; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P27" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO data item</t>
+        </is>
+      </c>
+      <c r="Q27" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="33" t="inlineStr">
@@ -6953,7 +7174,7 @@
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/ResourceEfficiencyDatum</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000028</t>
         </is>
       </c>
       <c r="E28" s="33" t="inlineStr">
@@ -6963,12 +7184,12 @@
       </c>
       <c r="F28" s="33" t="inlineStr">
         <is>
-          <t>IAO data item (IAO_0000027)</t>
+          <t>IAO data item (http://purl.obolibrary.org/obo/IAO_0000027)</t>
         </is>
       </c>
       <c r="G28" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — the class is a calculated/result datum, not an intrinsic universal ‘efficiency’.</t>
+          <t>ACCEPT ? calculated result datum, not an intrinsic efficiency quality.</t>
         </is>
       </c>
       <c r="H28" s="33" t="inlineStr">
@@ -6978,22 +7199,41 @@
       </c>
       <c r="I28" s="33" t="inlineStr">
         <is>
-          <t>ResourceEfficiencyDatum SubClassOf IAO data item.</t>
+          <t>MATSUS_0000028 SubClassOf IAO_0000027.</t>
         </is>
       </c>
       <c r="J28" s="33" t="inlineStr">
         <is>
-          <t>Later: represent numerator/output, resource input, method, boundary, unit and time interval.</t>
+          <t>Later: model numerator/output, resource input, method, boundary, unit, time interval, and calculation relations.</t>
         </is>
       </c>
       <c r="K28" s="33" t="n"/>
       <c r="L28" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M28" s="33" t="n"/>
-      <c r="N28" s="33" t="n"/>
+      <c r="N28" s="33" t="inlineStr">
+        <is>
+          <t>This is a calculated result datum, not an intrinsic efficiency quality.</t>
+        </is>
+      </c>
+      <c r="O28" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000205; SRC-001 Circular Berlin; UNEP domain meaning; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P28" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO data item</t>
+        </is>
+      </c>
+      <c r="Q28" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="33" t="inlineStr">
@@ -7013,7 +7253,7 @@
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MaterialResourceEfficiencyDatum</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000029</t>
         </is>
       </c>
       <c r="E29" s="33" t="inlineStr">
@@ -7023,12 +7263,12 @@
       </c>
       <c r="F29" s="33" t="inlineStr">
         <is>
-          <t>MatSus resource efficiency datum</t>
+          <t>MatSus resource efficiency datum (https://w3id.org/pmd/matsus/MATSUS_0000028)</t>
         </is>
       </c>
       <c r="G29" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — clear material-input specialization.</t>
+          <t>ACCEPT ? clear material-input specialization.</t>
         </is>
       </c>
       <c r="H29" s="33" t="inlineStr">
@@ -7038,22 +7278,41 @@
       </c>
       <c r="I29" s="33" t="inlineStr">
         <is>
-          <t>MaterialResourceEfficiencyDatum SubClassOf ResourceEfficiencyDatum.</t>
+          <t>MATSUS_0000029 SubClassOf MATSUS_0000028.</t>
         </is>
       </c>
       <c r="J29" s="33" t="inlineStr">
         <is>
-          <t>Later: constrain the stated resource input to a material quantity through the instance pattern.</t>
+          <t>Later: constrain the stated resource input to a material quantity and add method, unit, or boundary relations only through an approved pattern.</t>
         </is>
       </c>
       <c r="K29" s="33" t="n"/>
       <c r="L29" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M29" s="33" t="n"/>
-      <c r="N29" s="33" t="n"/>
+      <c r="N29" s="33" t="inlineStr">
+        <is>
+          <t>Material-input specialization of resource efficiency datum; no additional restriction is asserted in Batch 3.</t>
+        </is>
+      </c>
+      <c r="O29" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000137; SRC-003 European Environment Agency; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P29" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of resource efficiency datum</t>
+        </is>
+      </c>
+      <c r="Q29" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="33" t="inlineStr">
@@ -7073,7 +7332,7 @@
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/MetricSpecification</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000027</t>
         </is>
       </c>
       <c r="E30" s="33" t="inlineStr">
@@ -7083,12 +7342,12 @@
       </c>
       <c r="F30" s="33" t="inlineStr">
         <is>
-          <t>IAO directive information entity (IAO_0000033)</t>
+          <t>IAO directive information entity (http://purl.obolibrary.org/obo/IAO_0000033)</t>
         </is>
       </c>
       <c r="G30" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — a metric specification prescribes calculation inputs/methods; the resulting metric value remains a data item.</t>
+          <t>ACCEPT ? metric specifications prescribe calculation inputs and methods; resulting metric values remain data items.</t>
         </is>
       </c>
       <c r="H30" s="33" t="inlineStr">
@@ -7098,22 +7357,41 @@
       </c>
       <c r="I30" s="33" t="inlineStr">
         <is>
-          <t>MetricSpecification SubClassOf IAO directive information entity.</t>
+          <t>MATSUS_0000027 SubClassOf IAO_0000033.</t>
         </is>
       </c>
       <c r="J30" s="33" t="inlineStr">
         <is>
-          <t>Later: add prescribed quantities, calculation method, units, boundary and interpretation relations.</t>
+          <t>Later: relate prescribed quantities, calculation method, units, boundary, interpretation, and resulting datum.</t>
         </is>
       </c>
       <c r="K30" s="33" t="n"/>
       <c r="L30" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M30" s="33" t="n"/>
-      <c r="N30" s="33" t="n"/>
+      <c r="N30" s="33" t="inlineStr">
+        <is>
+          <t>Metric specifications prescribe methods; resulting metric values remain data items. No further logical restrictions are asserted in Batch 3.</t>
+        </is>
+      </c>
+      <c r="O30" s="33" t="inlineStr">
+        <is>
+          <t>ADD-SCO-012; SCO; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P30" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO directive information entity</t>
+        </is>
+      </c>
+      <c r="Q30" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="33" t="inlineStr">
@@ -7148,7 +7426,7 @@
       </c>
       <c r="G31" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT PROVISIONALLY — usable local specialization, but the current directive-only parent/definition may be too narrow if PMDco issue #488 adopts a descriptive-or-directive specification-document pattern.</t>
+          <t>EXTERNAL_ISSUE_DEPENDENT ? await PMDco #488; if the generic DesignSpecification proposal is rejected, reconsider a local MatSus class.</t>
         </is>
       </c>
       <c r="H31" s="33" t="inlineStr">
@@ -7158,12 +7436,12 @@
       </c>
       <c r="I31" s="33" t="inlineStr">
         <is>
-          <t>For now: CircularDesignSpecification SubClassOf IAO directive information entity.</t>
+          <t>No MatSus axiom in Batch 3.</t>
         </is>
       </c>
       <c r="J31" s="33" t="inlineStr">
         <is>
-          <t>After #488: reparent to PMDco DesignSpecification and revise the definition if PMDco adopts the mixed descriptive/directive scope.</t>
+          <t>Await PMDco #488 before local reconsideration.</t>
         </is>
       </c>
       <c r="K31" s="33" t="inlineStr">
@@ -7173,11 +7451,20 @@
       </c>
       <c r="L31" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>NOT IMPLEMENTED ? EXTERNAL ISSUE DEPENDENT</t>
         </is>
       </c>
       <c r="M31" s="33" t="n"/>
-      <c r="N31" s="33" t="n"/>
+      <c r="N31" s="33" t="inlineStr">
+        <is>
+          <t>Deferred pending PMDco #488.</t>
+        </is>
+      </c>
+      <c r="Q31" s="33" t="inlineStr">
+        <is>
+          <t>CONFIRMED ABSENT FROM MATSUS-EDIT 2026-09-07.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="33" t="inlineStr">
@@ -7197,7 +7484,7 @@
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/Modularity</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000038</t>
         </is>
       </c>
       <c r="E32" s="33" t="inlineStr">
@@ -7207,12 +7494,12 @@
       </c>
       <c r="F32" s="33" t="inlineStr">
         <is>
-          <t>BFO quality (BFO_0000019)</t>
+          <t>BFO quality (http://purl.obolibrary.org/obo/BFO_0000019)</t>
         </is>
       </c>
       <c r="G32" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — degree of modular organization is appropriately represented as a quality.</t>
+          <t>ACCEPT ? degree of modular organization is appropriately represented as a quality.</t>
         </is>
       </c>
       <c r="H32" s="33" t="inlineStr">
@@ -7222,22 +7509,41 @@
       </c>
       <c r="I32" s="33" t="inlineStr">
         <is>
-          <t>Modularity SubClassOf BFO quality.</t>
+          <t>MATSUS_0000038 SubClassOf BFO_0000019.</t>
         </is>
       </c>
       <c r="J32" s="33" t="inlineStr">
         <is>
-          <t>Later: add bearer and measurement datum/method only when a modularity metric is selected.</t>
+          <t>Later: model the bearer, measurement datum, degree, method, and any device- or design-specific subclasses.</t>
         </is>
       </c>
       <c r="K32" s="33" t="n"/>
       <c r="L32" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M32" s="33" t="n"/>
-      <c r="N32" s="33" t="n"/>
+      <c r="N32" s="33" t="inlineStr">
+        <is>
+          <t>Modularity is a dependent quality of a bearer, not an object aggregate.</t>
+        </is>
+      </c>
+      <c r="O32" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000146; SRC-002 Ellen MacArthur Foundation; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P32" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of BFO quality</t>
+        </is>
+      </c>
+      <c r="Q32" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="33" t="inlineStr">
@@ -7272,7 +7578,7 @@
       </c>
       <c r="G33" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT PROVISIONALLY — generic process parent is safe, but LOG alignment should be revisited before strengthening the hierarchy.</t>
+          <t>DEFER ? dedicated analysis of LOG transport, material-location-change, logistics, and material-flow-datum patterns is required.</t>
         </is>
       </c>
       <c r="H33" s="33" t="inlineStr">
@@ -7282,12 +7588,12 @@
       </c>
       <c r="I33" s="33" t="inlineStr">
         <is>
-          <t>MaterialFlowProcess SubClassOf BFO process.</t>
+          <t>No MatSus axiom in Batch 3.</t>
         </is>
       </c>
       <c r="J33" s="33" t="inlineStr">
         <is>
-          <t>Later: represent source/destination location or agent, moving material and relation to transport/transformation processes.</t>
+          <t>Resolve process-versus-datum semantics and LOG ownership before implementation.</t>
         </is>
       </c>
       <c r="K33" s="33" t="inlineStr">
@@ -7297,11 +7603,20 @@
       </c>
       <c r="L33" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>DEFERRED ? NOT IN BATCH 3</t>
         </is>
       </c>
       <c r="M33" s="33" t="n"/>
-      <c r="N33" s="33" t="n"/>
+      <c r="N33" s="33" t="inlineStr">
+        <is>
+          <t>Material-flow modelling remains outside Batch 3.</t>
+        </is>
+      </c>
+      <c r="Q33" s="33" t="inlineStr">
+        <is>
+          <t>CONFIRMED ABSENT FROM MATSUS-EDIT 2026-09-07.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="33" t="inlineStr">
@@ -7336,7 +7651,7 @@
       </c>
       <c r="G34" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT PROVISIONALLY — correct material-specific specialization of the provisional flow process.</t>
+          <t>DEFER ? parent and LOG boundary remain unsettled.</t>
         </is>
       </c>
       <c r="H34" s="33" t="inlineStr">
@@ -7346,12 +7661,12 @@
       </c>
       <c r="I34" s="33" t="inlineStr">
         <is>
-          <t>TextileMaterialFlowProcess SubClassOf MaterialFlowProcess.</t>
+          <t>No MatSus axiom in Batch 3.</t>
         </is>
       </c>
       <c r="J34" s="33" t="inlineStr">
         <is>
-          <t>Later: add textile participant constraints only after the generic material-flow/LOG pattern is settled.</t>
+          <t>Defer with MaterialFlowProcess.</t>
         </is>
       </c>
       <c r="K34" s="33" t="inlineStr">
@@ -7361,11 +7676,20 @@
       </c>
       <c r="L34" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>DEFERRED ? NOT IN BATCH 3</t>
         </is>
       </c>
       <c r="M34" s="33" t="n"/>
-      <c r="N34" s="33" t="n"/>
+      <c r="N34" s="33" t="inlineStr">
+        <is>
+          <t>TextileMaterialFlowProcess remains outside Batch 3 with its unsettled parent.</t>
+        </is>
+      </c>
+      <c r="Q34" s="33" t="inlineStr">
+        <is>
+          <t>CONFIRMED ABSENT FROM MATSUS-EDIT 2026-09-07.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="92" customHeight="1">
       <c r="A35" s="33" t="inlineStr">
@@ -7385,22 +7709,22 @@
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
-          <t>https://w3id.org/pmd/matsus/VirginMaterial</t>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000030</t>
         </is>
       </c>
       <c r="E35" s="33" t="inlineStr">
         <is>
-          <t>A material produced entirely from primary raw materials and containing no recovered or recycled material.</t>
+          <t>A material that has never been processed into any form of an end-use product.</t>
         </is>
       </c>
       <c r="F35" s="33" t="inlineStr">
         <is>
-          <t>PMDco material (PMD_0000000)</t>
+          <t>PMDco material (https://w3id.org/pmd/co/PMD_0000000)</t>
         </is>
       </c>
       <c r="G35" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT — a positive provenance/composition class is preferable to modelling non-virgin material as its logical complement.</t>
+          <t>ACCEPT ? ISO-grounded positive definition approved; use existing SecondaryMaterial and do not define a complement class.</t>
         </is>
       </c>
       <c r="H35" s="33" t="inlineStr">
@@ -7410,24 +7734,39 @@
       </c>
       <c r="I35" s="33" t="inlineStr">
         <is>
-          <t>VirginMaterial SubClassOf PMDco material.</t>
+          <t>MATSUS_0000030 SubClassOf PMD_0000000.</t>
         </is>
       </c>
       <c r="J35" s="33" t="inlineStr">
         <is>
-          <t>Later: use positive recycled/recovered-content assertions and a composition pattern; no complement axiom.</t>
+          <t>Later: add recovered-content, composition, and proportion axioms only from an approved competency query.</t>
         </is>
       </c>
       <c r="K35" s="33" t="n"/>
       <c r="L35" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
         </is>
       </c>
       <c r="M35" s="33" t="n"/>
       <c r="N35" s="33" t="inlineStr">
         <is>
-          <t>‘Non-virgin material’ is an informal umbrella covering recovered material, recycled material, secondary material, and materials containing some proportion of such content. It is not modelled as the OWL complement of virgin material because mixed content is common and absence of virgin status cannot be inferred under the open-world assumption.</t>
+          <t>Use the existing positive SecondaryMaterial class MATSUS_0000003. Do not create NonVirginMaterial or model non-virgin material as the complement of VirginMaterial.</t>
+        </is>
+      </c>
+      <c r="O35" s="33" t="inlineStr">
+        <is>
+          <t>MKB-000150; SRC-002 Ellen MacArthur Foundation; ISO 21067-2:2015 terminology as reproduced in ISO/DIS 15270-1; Batch 3 planning report.</t>
+        </is>
+      </c>
+      <c r="P35" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of PMDco material</t>
+        </is>
+      </c>
+      <c r="Q35" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
     </row>
@@ -7464,7 +7803,7 @@
       </c>
       <c r="G36" s="33" t="inlineStr">
         <is>
-          <t>ACCEPT PROVISIONALLY — role modelling is correct and the LOG parent is reasonable; PMDco issue #486 may provide the upstream class and require reconciliation.</t>
+          <t>EXTERNAL_ISSUE_DEPENDENT ? await PMDco #486; reuse upstream if accepted, otherwise reconsider a local MatSus class.</t>
         </is>
       </c>
       <c r="H36" s="33" t="inlineStr">
@@ -7474,12 +7813,12 @@
       </c>
       <c r="I36" s="33" t="inlineStr">
         <is>
-          <t>For now: FeedstockRole SubClassOf LOG material resource role.</t>
+          <t>No MatSus axiom in Batch 3.</t>
         </is>
       </c>
       <c r="J36" s="33" t="inlineStr">
         <is>
-          <t>Later: add bearer/realized-in/process-input relations only after the PMDco/LOG placement decision.</t>
+          <t>Await PMDco #486 and its PMDco/LOG placement decision.</t>
         </is>
       </c>
       <c r="K36" s="33" t="inlineStr">
@@ -7489,11 +7828,20 @@
       </c>
       <c r="L36" s="33" t="inlineStr">
         <is>
-          <t>DRAFT EXISTS; NOT IN CURRENT SOURCE</t>
+          <t>NOT IMPLEMENTED ? EXTERNAL ISSUE DEPENDENT</t>
         </is>
       </c>
       <c r="M36" s="33" t="n"/>
-      <c r="N36" s="33" t="n"/>
+      <c r="N36" s="33" t="inlineStr">
+        <is>
+          <t>Deferred pending PMDco #486.</t>
+        </is>
+      </c>
+      <c r="Q36" s="33" t="inlineStr">
+        <is>
+          <t>CONFIRMED ABSENT FROM MATSUS-EDIT 2026-09-07.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="42" customHeight="1">
       <c r="A37" s="33" t="inlineStr">
@@ -8187,6 +8535,89 @@
       <c r="N46" s="33" t="inlineStr">
         <is>
           <t>Example: reduce virgin aluminium input by 20% relative to the 2025 baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="58" customHeight="1">
+      <c r="A47" s="33" t="inlineStr">
+        <is>
+          <t>Human-gate refinement derived from MKB-000184 review</t>
+        </is>
+      </c>
+      <c r="B47" s="33" t="inlineStr">
+        <is>
+          <t>MatSus</t>
+        </is>
+      </c>
+      <c r="C47" s="33" t="inlineStr">
+        <is>
+          <t>refusal strategy specification</t>
+        </is>
+      </c>
+      <c r="D47" s="33" t="inlineStr">
+        <is>
+          <t>https://w3id.org/pmd/matsus/MATSUS_0000039</t>
+        </is>
+      </c>
+      <c r="E47" s="33" t="inlineStr">
+        <is>
+          <t>A plan specification that prescribes product, packaging, or service features intended to enable or encourage a refusal process and thereby avoid material use or waste generation.</t>
+        </is>
+      </c>
+      <c r="F47" s="33" t="inlineStr">
+        <is>
+          <t>IAO plan specification (http://purl.obolibrary.org/obo/IAO_0000104)</t>
+        </is>
+      </c>
+      <c r="G47" s="33" t="inlineStr">
+        <is>
+          <t>ACCEPT ? human-gate modelling refinement; plan specification distinct from the actual refusal occurrence.</t>
+        </is>
+      </c>
+      <c r="H47" s="33" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I47" s="33" t="inlineStr">
+        <is>
+          <t>MATSUS_0000039 SubClassOf IAO_0000104.</t>
+        </is>
+      </c>
+      <c r="J47" s="33" t="inlineStr">
+        <is>
+          <t>Later: relate to refusal processes, resource-input-reduction objectives, design specifications, affected product features, and realization. No logical relation to RefusalProcess in Batch 3.</t>
+        </is>
+      </c>
+      <c r="K47" s="33" t="n"/>
+      <c r="L47" s="33" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED IN MATSUS-EDIT (MKB1 IR2 BATCH 3)</t>
+        </is>
+      </c>
+      <c r="M47" s="33" t="inlineStr">
+        <is>
+          <t>Additional human-gate modelling refinement; not a seventeenth original source candidate.</t>
+        </is>
+      </c>
+      <c r="N47" s="33" t="inlineStr">
+        <is>
+          <t>Examples are recorded in the ontology rdfs:comment. This human-gate addition remains separate from RefusalProcess; all process/specification relations are deferred.</t>
+        </is>
+      </c>
+      <c r="O47" s="33" t="inlineStr">
+        <is>
+          <t>Human-gate modelling refinement derived from the MKB-000184 RefusalProcess review and the 2026-09-04 Batch 3 review; not an original MKB source candidate.</t>
+        </is>
+      </c>
+      <c r="P47" s="33" t="inlineStr">
+        <is>
+          <t>new MatSus subclass of IAO plan specification</t>
+        </is>
+      </c>
+      <c r="Q47" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATED 2026-09-07 ? Functional Syntax parsing, catalog merge, ODK-compatible full build with ROBOT 1.9.10, ELK consistency, local and merged OWL 2 DL, ID policy, exact declarations, parents, annotations and logical axioms, imports, and all five repository SPARQL checks pass; ROBOT report has 58 warnings versus 45 on main, with the +13 exactly the expected missing_definition rule mismatch for English SKOS definitions.</t>
         </is>
       </c>
     </row>

</xml_diff>